<commit_message>
JIM001 v4.1: add payment doc, dates, and gross columns to monthly open sheet.
Extend the Open Invoices by Month builder and regenerated workbook with payment reference and cash detail from insights and payments.csv.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/analysis/debtors/JIM001/reports/JIM001_LPG_Reconciliation_v4.1.xlsx
+++ b/analysis/debtors/JIM001/reports/JIM001_LPG_Reconciliation_v4.1.xlsx
@@ -18244,17 +18244,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:K83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -18288,20 +18291,35 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Payments Allocated</t>
+          <t>Payment Doc #</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>Payment Date(s)</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Payment Gross (Original)</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Payment Allocated (Month)</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
           <t>Open Invoices (Sum)</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Month Status</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>LPG Invoice Doc Count</t>
         </is>
@@ -18324,19 +18342,32 @@
       <c r="D4" s="6" t="n">
         <v>9000.02</v>
       </c>
-      <c r="E4" s="6" t="n">
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>00004904</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>2019-01-21</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>7000.0</v>
+      </c>
+      <c r="H4" s="6" t="n">
         <v>6556.68</v>
       </c>
-      <c r="F4" s="6" t="n">
+      <c r="I4" s="6" t="n">
         <v>2443.34</v>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="H4" s="6" t="n">
-        <v>2</v>
+      <c r="K4" s="6" t="n">
+        <v>2.0</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
@@ -18356,19 +18387,34 @@
       <c r="D5" s="6" t="n">
         <v>19306.77</v>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="I5" s="6" t="n">
         <v>19306.77</v>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="H5" s="6" t="n">
-        <v>19</v>
+      <c r="K5" s="6" t="n">
+        <v>19.0</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
@@ -18388,19 +18434,32 @@
       <c r="D6" s="6" t="n">
         <v>10097.41</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>00005437</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>2019-04-24</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="n">
         <v>9925.0</v>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="H6" s="6" t="n">
+        <v>9925.0</v>
+      </c>
+      <c r="I6" s="6" t="n">
         <v>172.41</v>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="H6" s="6" t="n">
-        <v>11</v>
+      <c r="K6" s="6" t="n">
+        <v>11.0</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -18420,19 +18479,34 @@
       <c r="D7" s="6" t="n">
         <v>4374.98</v>
       </c>
-      <c r="E7" s="6" t="n">
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="I7" s="6" t="n">
         <v>4374.98</v>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="H7" s="6" t="n">
-        <v>14</v>
+      <c r="K7" s="6" t="n">
+        <v>14.0</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
@@ -18452,19 +18526,32 @@
       <c r="D8" s="6" t="n">
         <v>13504.86</v>
       </c>
-      <c r="E8" s="6" t="n">
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>00005436</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>2019-05-06</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>13505.0</v>
+      </c>
+      <c r="H8" s="6" t="n">
         <v>13504.86</v>
       </c>
-      <c r="F8" s="6" t="n">
+      <c r="I8" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H8" s="6" t="n">
-        <v>9</v>
+      <c r="K8" s="6" t="n">
+        <v>9.0</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
@@ -18484,19 +18571,32 @@
       <c r="D9" s="6" t="n">
         <v>8710.63</v>
       </c>
-      <c r="E9" s="6" t="n">
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>00005618</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>2019-06-20</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="n">
         <v>8625.0</v>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="H9" s="6" t="n">
+        <v>8625.0</v>
+      </c>
+      <c r="I9" s="6" t="n">
         <v>85.63</v>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="H9" s="6" t="n">
-        <v>6</v>
+      <c r="K9" s="6" t="n">
+        <v>6.0</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -18516,19 +18616,32 @@
       <c r="D10" s="6" t="n">
         <v>12750.0</v>
       </c>
-      <c r="E10" s="6" t="n">
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>00005804</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>2019-07-04</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="n">
         <v>12750.0</v>
       </c>
-      <c r="F10" s="6" t="n">
+      <c r="H10" s="6" t="n">
+        <v>12750.0</v>
+      </c>
+      <c r="I10" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H10" s="6" t="n">
-        <v>9</v>
+      <c r="K10" s="6" t="n">
+        <v>9.0</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
@@ -18548,19 +18661,32 @@
       <c r="D11" s="6" t="n">
         <v>14981.01</v>
       </c>
-      <c r="E11" s="6" t="n">
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>00005876</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>2019-08-06</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="n">
         <v>14429.0</v>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="H11" s="6" t="n">
+        <v>14429.0</v>
+      </c>
+      <c r="I11" s="6" t="n">
         <v>552.01</v>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="H11" s="6" t="n">
-        <v>11</v>
+      <c r="K11" s="6" t="n">
+        <v>11.0</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
@@ -18580,19 +18706,32 @@
       <c r="D12" s="6" t="n">
         <v>13874.99</v>
       </c>
-      <c r="E12" s="6" t="n">
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>00005988</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>2019-09-04</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>13875.0</v>
+      </c>
+      <c r="H12" s="6" t="n">
         <v>13874.99</v>
       </c>
-      <c r="F12" s="6" t="n">
+      <c r="I12" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H12" s="6" t="n">
-        <v>10</v>
+      <c r="K12" s="6" t="n">
+        <v>10.0</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
@@ -18612,19 +18751,32 @@
       <c r="D13" s="6" t="n">
         <v>13322.98</v>
       </c>
-      <c r="E13" s="6" t="n">
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>00006104</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>2019-10-21</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>13875.0</v>
+      </c>
+      <c r="H13" s="6" t="n">
         <v>13874.98</v>
       </c>
-      <c r="F13" s="6" t="n">
+      <c r="I13" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>OVERPAID</t>
         </is>
       </c>
-      <c r="H13" s="6" t="n">
-        <v>9</v>
+      <c r="K13" s="6" t="n">
+        <v>9.0</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
@@ -18644,19 +18796,32 @@
       <c r="D14" s="6" t="n">
         <v>10874.96</v>
       </c>
-      <c r="E14" s="6" t="n">
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>00006316</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>2019-12-09</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>10875.0</v>
+      </c>
+      <c r="H14" s="6" t="n">
         <v>10874.96</v>
       </c>
-      <c r="F14" s="6" t="n">
+      <c r="I14" s="6" t="n">
         <v>-0.0</v>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H14" s="6" t="n">
-        <v>7</v>
+      <c r="K14" s="6" t="n">
+        <v>7.0</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -18676,19 +18841,32 @@
       <c r="D15" s="6" t="n">
         <v>12914.93</v>
       </c>
-      <c r="E15" s="6" t="n">
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>00006376</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>2019-12-27</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>12915.0</v>
+      </c>
+      <c r="H15" s="6" t="n">
         <v>12914.93</v>
       </c>
-      <c r="F15" s="6" t="n">
+      <c r="I15" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="J15" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H15" s="6" t="n">
-        <v>11</v>
+      <c r="K15" s="6" t="n">
+        <v>11.0</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
@@ -18708,19 +18886,32 @@
       <c r="D16" s="6" t="n">
         <v>12731.05</v>
       </c>
-      <c r="E16" s="6" t="n">
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>00006423</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>2020-01-17</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="n">
         <v>12715.0</v>
       </c>
-      <c r="F16" s="6" t="n">
+      <c r="H16" s="6" t="n">
+        <v>12715.0</v>
+      </c>
+      <c r="I16" s="6" t="n">
         <v>16.05</v>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="H16" s="6" t="n">
-        <v>8</v>
+      <c r="K16" s="6" t="n">
+        <v>8.0</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
@@ -18740,19 +18931,32 @@
       <c r="D17" s="6" t="n">
         <v>15302.89</v>
       </c>
-      <c r="E17" s="6" t="n">
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>00006685</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>2020-03-03</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="n">
         <v>15302.8</v>
       </c>
-      <c r="F17" s="6" t="n">
+      <c r="H17" s="6" t="n">
+        <v>15302.8</v>
+      </c>
+      <c r="I17" s="6" t="n">
         <v>0.09</v>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="J17" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="H17" s="6" t="n">
-        <v>10</v>
+      <c r="K17" s="6" t="n">
+        <v>10.0</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
@@ -18772,19 +18976,34 @@
       <c r="D18" s="6" t="n">
         <v>11250.03</v>
       </c>
-      <c r="E18" s="6" t="n">
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="F18" s="6" t="n">
+      <c r="I18" s="6" t="n">
         <v>11250.03</v>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="J18" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="H18" s="6" t="n">
-        <v>8</v>
+      <c r="K18" s="6" t="n">
+        <v>8.0</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
@@ -18804,19 +19023,34 @@
       <c r="D19" s="6" t="n">
         <v>10125.03</v>
       </c>
-      <c r="E19" s="6" t="n">
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="F19" s="6" t="n">
+      <c r="I19" s="6" t="n">
         <v>10125.03</v>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="J19" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="H19" s="6" t="n">
-        <v>7</v>
+      <c r="K19" s="6" t="n">
+        <v>7.0</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
@@ -18836,19 +19070,32 @@
       <c r="D20" s="6" t="n">
         <v>12518.2</v>
       </c>
-      <c r="E20" s="6" t="n">
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>00008420</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>2021-04-09</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>12518.21</v>
+      </c>
+      <c r="H20" s="6" t="n">
         <v>12518.2</v>
       </c>
-      <c r="F20" s="6" t="n">
+      <c r="I20" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="J20" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H20" s="6" t="n">
-        <v>7</v>
+      <c r="K20" s="6" t="n">
+        <v>7.0</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
@@ -18868,19 +19115,32 @@
       <c r="D21" s="6" t="n">
         <v>9765.76</v>
       </c>
-      <c r="E21" s="6" t="n">
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>00008764</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>2021-05-11</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="n">
         <v>9765.76</v>
       </c>
-      <c r="F21" s="6" t="n">
+      <c r="H21" s="6" t="n">
+        <v>9765.76</v>
+      </c>
+      <c r="I21" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="J21" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H21" s="6" t="n">
-        <v>7</v>
+      <c r="K21" s="6" t="n">
+        <v>7.0</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -18900,19 +19160,32 @@
       <c r="D22" s="6" t="n">
         <v>12222.9</v>
       </c>
-      <c r="E22" s="6" t="n">
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>00009315</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>2021-06-03</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="n">
         <v>12222.9</v>
       </c>
-      <c r="F22" s="6" t="n">
+      <c r="H22" s="6" t="n">
+        <v>12222.9</v>
+      </c>
+      <c r="I22" s="6" t="n">
         <v>-0.0</v>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="J22" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H22" s="6" t="n">
-        <v>9</v>
+      <c r="K22" s="6" t="n">
+        <v>9.0</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
@@ -18932,19 +19205,32 @@
       <c r="D23" s="6" t="n">
         <v>11292.11</v>
       </c>
-      <c r="E23" s="6" t="n">
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>00009996</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="n">
         <v>11292.11</v>
       </c>
-      <c r="F23" s="6" t="n">
+      <c r="H23" s="6" t="n">
+        <v>11292.11</v>
+      </c>
+      <c r="I23" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="J23" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H23" s="6" t="n">
-        <v>8</v>
+      <c r="K23" s="6" t="n">
+        <v>8.0</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
@@ -18964,19 +19250,32 @@
       <c r="D24" s="6" t="n">
         <v>9079.94</v>
       </c>
-      <c r="E24" s="6" t="n">
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>00010226</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>2021-08-05</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="n">
         <v>9079.94</v>
       </c>
-      <c r="F24" s="6" t="n">
+      <c r="H24" s="6" t="n">
+        <v>9079.94</v>
+      </c>
+      <c r="I24" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="J24" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H24" s="6" t="n">
-        <v>7</v>
+      <c r="K24" s="6" t="n">
+        <v>7.0</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
@@ -18996,19 +19295,32 @@
       <c r="D25" s="6" t="n">
         <v>13012.51</v>
       </c>
-      <c r="E25" s="6" t="n">
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>00010584</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>2021-09-02</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="n">
         <v>13012.5</v>
       </c>
-      <c r="F25" s="6" t="n">
+      <c r="H25" s="6" t="n">
+        <v>13012.5</v>
+      </c>
+      <c r="I25" s="6" t="n">
         <v>0.01</v>
       </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="J25" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H25" s="6" t="n">
-        <v>15</v>
+      <c r="K25" s="6" t="n">
+        <v>15.0</v>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
@@ -19028,19 +19340,32 @@
       <c r="D26" s="6" t="n">
         <v>13260.28</v>
       </c>
-      <c r="E26" s="6" t="n">
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>00011068</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>2021-10-07</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="n">
         <v>13260.28</v>
       </c>
-      <c r="F26" s="6" t="n">
+      <c r="H26" s="6" t="n">
+        <v>13260.28</v>
+      </c>
+      <c r="I26" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="J26" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H26" s="6" t="n">
-        <v>11</v>
+      <c r="K26" s="6" t="n">
+        <v>11.0</v>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
@@ -19060,19 +19385,32 @@
       <c r="D27" s="6" t="n">
         <v>13329.62</v>
       </c>
-      <c r="E27" s="6" t="n">
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>00011558</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>2021-11-04</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="n">
         <v>12929.71</v>
       </c>
-      <c r="F27" s="6" t="n">
+      <c r="H27" s="6" t="n">
+        <v>12929.71</v>
+      </c>
+      <c r="I27" s="6" t="n">
         <v>399.91</v>
       </c>
-      <c r="G27" s="5" t="inlineStr">
+      <c r="J27" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="H27" s="6" t="n">
-        <v>11</v>
+      <c r="K27" s="6" t="n">
+        <v>11.0</v>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
@@ -19092,19 +19430,32 @@
       <c r="D28" s="6" t="n">
         <v>16378.91</v>
       </c>
-      <c r="E28" s="6" t="n">
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>00012719</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>2022-01-31</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>17018.3</v>
+      </c>
+      <c r="H28" s="6" t="n">
         <v>16778.82</v>
       </c>
-      <c r="F28" s="6" t="n">
+      <c r="I28" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="J28" s="5" t="inlineStr">
         <is>
           <t>OVERPAID</t>
         </is>
       </c>
-      <c r="H28" s="6" t="n">
-        <v>10</v>
+      <c r="K28" s="6" t="n">
+        <v>10.0</v>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
@@ -19124,19 +19475,32 @@
       <c r="D29" s="6" t="n">
         <v>12399.78</v>
       </c>
-      <c r="E29" s="6" t="n">
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>00012146</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>2021-12-20</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="n">
         <v>12160.3</v>
       </c>
-      <c r="F29" s="6" t="n">
+      <c r="H29" s="6" t="n">
+        <v>12160.3</v>
+      </c>
+      <c r="I29" s="6" t="n">
         <v>239.48</v>
       </c>
-      <c r="G29" s="5" t="inlineStr">
+      <c r="J29" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="H29" s="6" t="n">
-        <v>6</v>
+      <c r="K29" s="6" t="n">
+        <v>6.0</v>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
@@ -19156,19 +19520,32 @@
       <c r="D30" s="6" t="n">
         <v>14982.58</v>
       </c>
-      <c r="E30" s="6" t="n">
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>00013245</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>2022-03-17</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="n">
         <v>14982.58</v>
       </c>
-      <c r="F30" s="6" t="n">
+      <c r="H30" s="6" t="n">
+        <v>14982.58</v>
+      </c>
+      <c r="I30" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G30" s="5" t="inlineStr">
+      <c r="J30" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H30" s="6" t="n">
-        <v>7</v>
+      <c r="K30" s="6" t="n">
+        <v>7.0</v>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
@@ -19188,19 +19565,32 @@
       <c r="D31" s="6" t="n">
         <v>13949.0</v>
       </c>
-      <c r="E31" s="6" t="n">
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>00013583</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>2022-04-12</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="n">
         <v>13949.0</v>
       </c>
-      <c r="F31" s="6" t="n">
+      <c r="H31" s="6" t="n">
+        <v>13949.0</v>
+      </c>
+      <c r="I31" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="J31" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H31" s="6" t="n">
-        <v>8</v>
+      <c r="K31" s="6" t="n">
+        <v>8.0</v>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
@@ -19220,19 +19610,34 @@
       <c r="D32" s="6" t="n">
         <v>14943.48</v>
       </c>
-      <c r="E32" s="6" t="n">
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="F32" s="6" t="n">
+      <c r="I32" s="6" t="n">
         <v>14943.48</v>
       </c>
-      <c r="G32" s="5" t="inlineStr">
+      <c r="J32" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="H32" s="6" t="n">
-        <v>8</v>
+      <c r="K32" s="6" t="n">
+        <v>8.0</v>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
@@ -19252,19 +19657,32 @@
       <c r="D33" s="6" t="n">
         <v>18184.64</v>
       </c>
-      <c r="E33" s="6" t="n">
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>00014135</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>2022-06-01</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="n">
         <v>18184.64</v>
       </c>
-      <c r="F33" s="6" t="n">
+      <c r="H33" s="6" t="n">
+        <v>18184.64</v>
+      </c>
+      <c r="I33" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G33" s="5" t="inlineStr">
+      <c r="J33" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H33" s="6" t="n">
-        <v>8</v>
+      <c r="K33" s="6" t="n">
+        <v>8.0</v>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
@@ -19284,19 +19702,32 @@
       <c r="D34" s="6" t="n">
         <v>18947.57</v>
       </c>
-      <c r="E34" s="6" t="n">
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>00015071</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>2022-07-26</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="n">
         <v>17275.67</v>
       </c>
-      <c r="F34" s="6" t="n">
+      <c r="H34" s="6" t="n">
+        <v>17275.67</v>
+      </c>
+      <c r="I34" s="6" t="n">
         <v>1671.9</v>
       </c>
-      <c r="G34" s="5" t="inlineStr">
+      <c r="J34" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="H34" s="6" t="n">
-        <v>9</v>
+      <c r="K34" s="6" t="n">
+        <v>9.0</v>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
@@ -19316,19 +19747,32 @@
       <c r="D35" s="6" t="n">
         <v>16103.76</v>
       </c>
-      <c r="E35" s="6" t="n">
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>00015473</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>2022-08-11</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="n">
         <v>14488.95</v>
       </c>
-      <c r="F35" s="6" t="n">
+      <c r="H35" s="6" t="n">
+        <v>14488.95</v>
+      </c>
+      <c r="I35" s="6" t="n">
         <v>1614.81</v>
       </c>
-      <c r="G35" s="5" t="inlineStr">
+      <c r="J35" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="H35" s="6" t="n">
-        <v>8</v>
+      <c r="K35" s="6" t="n">
+        <v>8.0</v>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
@@ -19348,19 +19792,32 @@
       <c r="D36" s="6" t="n">
         <v>17169.29</v>
       </c>
-      <c r="E36" s="6" t="n">
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>00015987</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>2022-09-10</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="n">
         <v>17169.29</v>
       </c>
-      <c r="F36" s="6" t="n">
+      <c r="H36" s="6" t="n">
+        <v>17169.29</v>
+      </c>
+      <c r="I36" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G36" s="5" t="inlineStr">
+      <c r="J36" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H36" s="6" t="n">
-        <v>5</v>
+      <c r="K36" s="6" t="n">
+        <v>5.0</v>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
@@ -19380,19 +19837,32 @@
       <c r="D37" s="6" t="n">
         <v>15337.5</v>
       </c>
-      <c r="E37" s="6" t="n">
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>00016648</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>2022-10-20</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="n">
+        <v>15885.27</v>
+      </c>
+      <c r="H37" s="6" t="n">
         <v>15337.5</v>
       </c>
-      <c r="F37" s="6" t="n">
+      <c r="I37" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G37" s="5" t="inlineStr">
+      <c r="J37" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H37" s="6" t="n">
-        <v>9</v>
+      <c r="K37" s="6" t="n">
+        <v>9.0</v>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
@@ -19412,19 +19882,32 @@
       <c r="D38" s="6" t="n">
         <v>16606.08</v>
       </c>
-      <c r="E38" s="6" t="n">
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>00017073</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>2022-11-24</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="n">
         <v>13838.4</v>
       </c>
-      <c r="F38" s="6" t="n">
+      <c r="H38" s="6" t="n">
+        <v>13838.4</v>
+      </c>
+      <c r="I38" s="6" t="n">
         <v>2767.68</v>
       </c>
-      <c r="G38" s="5" t="inlineStr">
+      <c r="J38" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="H38" s="6" t="n">
-        <v>5</v>
+      <c r="K38" s="6" t="n">
+        <v>5.0</v>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
@@ -19444,19 +19927,32 @@
       <c r="D39" s="6" t="n">
         <v>15222.24</v>
       </c>
-      <c r="E39" s="6" t="n">
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>00017578</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>2022-12-19</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="n">
+        <v>17989.92</v>
+      </c>
+      <c r="H39" s="6" t="n">
         <v>15222.24</v>
       </c>
-      <c r="F39" s="6" t="n">
+      <c r="I39" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G39" s="5" t="inlineStr">
+      <c r="J39" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H39" s="6" t="n">
-        <v>5</v>
+      <c r="K39" s="6" t="n">
+        <v>5.0</v>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1">
@@ -19476,19 +19972,32 @@
       <c r="D40" s="6" t="n">
         <v>8139.84</v>
       </c>
-      <c r="E40" s="6" t="n">
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>00017777</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>2023-01-19</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="n">
         <v>10825.92</v>
       </c>
-      <c r="F40" s="6" t="n">
+      <c r="H40" s="6" t="n">
+        <v>10825.92</v>
+      </c>
+      <c r="I40" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G40" s="5" t="inlineStr">
+      <c r="J40" s="5" t="inlineStr">
         <is>
           <t>OVERPAID</t>
         </is>
       </c>
-      <c r="H40" s="6" t="n">
-        <v>7</v>
+      <c r="K40" s="6" t="n">
+        <v>7.0</v>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
@@ -19508,19 +20017,32 @@
       <c r="D41" s="6" t="n">
         <v>27870.44</v>
       </c>
-      <c r="E41" s="6" t="n">
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>00018185</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>2023-02-13</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="n">
         <v>25184.36</v>
       </c>
-      <c r="F41" s="6" t="n">
+      <c r="H41" s="6" t="n">
+        <v>25184.36</v>
+      </c>
+      <c r="I41" s="6" t="n">
         <v>2686.08</v>
       </c>
-      <c r="G41" s="5" t="inlineStr">
+      <c r="J41" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="H41" s="6" t="n">
-        <v>9</v>
+      <c r="K41" s="6" t="n">
+        <v>9.0</v>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
@@ -19540,19 +20062,32 @@
       <c r="D42" s="6" t="n">
         <v>11335.68</v>
       </c>
-      <c r="E42" s="6" t="n">
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>00019176</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>2023-03-22</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="n">
         <v>11335.68</v>
       </c>
-      <c r="F42" s="6" t="n">
+      <c r="H42" s="6" t="n">
+        <v>11335.68</v>
+      </c>
+      <c r="I42" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G42" s="5" t="inlineStr">
+      <c r="J42" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H42" s="6" t="n">
-        <v>4</v>
+      <c r="K42" s="6" t="n">
+        <v>4.0</v>
       </c>
     </row>
     <row r="43" ht="20" customHeight="1">
@@ -19572,19 +20107,32 @@
       <c r="D43" s="6" t="n">
         <v>12343.07</v>
       </c>
-      <c r="E43" s="6" t="n">
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>00020357</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>2023-05-02</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="n">
         <v>12343.07</v>
       </c>
-      <c r="F43" s="6" t="n">
+      <c r="H43" s="6" t="n">
+        <v>12343.07</v>
+      </c>
+      <c r="I43" s="6" t="n">
         <v>-0.0</v>
       </c>
-      <c r="G43" s="5" t="inlineStr">
+      <c r="J43" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H43" s="6" t="n">
-        <v>3</v>
+      <c r="K43" s="6" t="n">
+        <v>3.0</v>
       </c>
     </row>
     <row r="44" ht="20" customHeight="1">
@@ -19604,19 +20152,32 @@
       <c r="D44" s="6" t="n">
         <v>16111.5</v>
       </c>
-      <c r="E44" s="6" t="n">
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>00021193</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>2023-05-31</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="n">
         <v>15409.46</v>
       </c>
-      <c r="F44" s="6" t="n">
+      <c r="H44" s="6" t="n">
+        <v>15409.46</v>
+      </c>
+      <c r="I44" s="6" t="n">
         <v>702.04</v>
       </c>
-      <c r="G44" s="5" t="inlineStr">
+      <c r="J44" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="H44" s="6" t="n">
-        <v>4</v>
+      <c r="K44" s="6" t="n">
+        <v>4.0</v>
       </c>
     </row>
     <row r="45" ht="20" customHeight="1">
@@ -19636,19 +20197,32 @@
       <c r="D45" s="6" t="n">
         <v>15140.69</v>
       </c>
-      <c r="E45" s="6" t="n">
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>00022711</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>2023-07-21</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="n">
         <v>15140.69</v>
       </c>
-      <c r="F45" s="6" t="n">
+      <c r="H45" s="6" t="n">
+        <v>15140.69</v>
+      </c>
+      <c r="I45" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G45" s="5" t="inlineStr">
+      <c r="J45" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H45" s="6" t="n">
-        <v>4</v>
+      <c r="K45" s="6" t="n">
+        <v>4.0</v>
       </c>
     </row>
     <row r="46" ht="20" customHeight="1">
@@ -19668,19 +20242,32 @@
       <c r="D46" s="6" t="n">
         <v>13806.77</v>
       </c>
-      <c r="E46" s="6" t="n">
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>00023280</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>2023-08-11</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="n">
         <v>13806.77</v>
       </c>
-      <c r="F46" s="6" t="n">
+      <c r="H46" s="6" t="n">
+        <v>13806.77</v>
+      </c>
+      <c r="I46" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G46" s="5" t="inlineStr">
+      <c r="J46" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H46" s="6" t="n">
-        <v>4</v>
+      <c r="K46" s="6" t="n">
+        <v>4.0</v>
       </c>
     </row>
     <row r="47" ht="20" customHeight="1">
@@ -19700,19 +20287,32 @@
       <c r="D47" s="6" t="n">
         <v>16964.84</v>
       </c>
-      <c r="E47" s="6" t="n">
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>00023977</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>2023-09-05</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="n">
         <v>16964.84</v>
       </c>
-      <c r="F47" s="6" t="n">
+      <c r="H47" s="6" t="n">
+        <v>16964.84</v>
+      </c>
+      <c r="I47" s="6" t="n">
         <v>-0.0</v>
       </c>
-      <c r="G47" s="5" t="inlineStr">
+      <c r="J47" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H47" s="6" t="n">
-        <v>5</v>
+      <c r="K47" s="6" t="n">
+        <v>5.0</v>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
@@ -19732,19 +20332,32 @@
       <c r="D48" s="6" t="n">
         <v>13911.54</v>
       </c>
-      <c r="E48" s="6" t="n">
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>00025394</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>2023-10-24</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="n">
         <v>13911.54</v>
       </c>
-      <c r="F48" s="6" t="n">
+      <c r="H48" s="6" t="n">
+        <v>13911.54</v>
+      </c>
+      <c r="I48" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G48" s="5" t="inlineStr">
+      <c r="J48" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H48" s="6" t="n">
-        <v>5</v>
+      <c r="K48" s="6" t="n">
+        <v>5.0</v>
       </c>
     </row>
     <row r="49" ht="20" customHeight="1">
@@ -19764,19 +20377,32 @@
       <c r="D49" s="6" t="n">
         <v>15766.57</v>
       </c>
-      <c r="E49" s="6" t="n">
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>00026601</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>2023-11-29</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="n">
         <v>12520.81</v>
       </c>
-      <c r="F49" s="6" t="n">
+      <c r="H49" s="6" t="n">
+        <v>12520.81</v>
+      </c>
+      <c r="I49" s="6" t="n">
         <v>3245.76</v>
       </c>
-      <c r="G49" s="5" t="inlineStr">
+      <c r="J49" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="H49" s="6" t="n">
-        <v>5</v>
+      <c r="K49" s="6" t="n">
+        <v>5.0</v>
       </c>
     </row>
     <row r="50" ht="20" customHeight="1">
@@ -19796,19 +20422,32 @@
       <c r="D50" s="6" t="n">
         <v>8026.98</v>
       </c>
-      <c r="E50" s="6" t="n">
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>00027468</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>2023-12-29</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="n">
+        <v>24801.28</v>
+      </c>
+      <c r="H50" s="6" t="n">
         <v>11272.74</v>
       </c>
-      <c r="F50" s="6" t="n">
+      <c r="I50" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G50" s="5" t="inlineStr">
+      <c r="J50" s="5" t="inlineStr">
         <is>
           <t>OVERPAID</t>
         </is>
       </c>
-      <c r="H50" s="6" t="n">
-        <v>6</v>
+      <c r="K50" s="6" t="n">
+        <v>6.0</v>
       </c>
     </row>
     <row r="51" ht="20" customHeight="1">
@@ -19828,19 +20467,32 @@
       <c r="D51" s="6" t="n">
         <v>13528.54</v>
       </c>
-      <c r="E51" s="6" t="n">
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>00030269</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>2024-04-24</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="n">
+        <v>16151.04</v>
+      </c>
+      <c r="H51" s="6" t="n">
         <v>13528.54</v>
       </c>
-      <c r="F51" s="6" t="n">
+      <c r="I51" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G51" s="5" t="inlineStr">
+      <c r="J51" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H51" s="6" t="n">
-        <v>5</v>
+      <c r="K51" s="6" t="n">
+        <v>5.0</v>
       </c>
     </row>
     <row r="52" ht="20" customHeight="1">
@@ -19860,19 +20512,32 @@
       <c r="D52" s="6" t="n">
         <v>11625.12</v>
       </c>
-      <c r="E52" s="6" t="n">
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>00028893</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>2024-02-20</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="n">
+        <v>14208.48</v>
+      </c>
+      <c r="H52" s="6" t="n">
         <v>11625.12</v>
       </c>
-      <c r="F52" s="6" t="n">
+      <c r="I52" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G52" s="5" t="inlineStr">
+      <c r="J52" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H52" s="6" t="n">
-        <v>3</v>
+      <c r="K52" s="6" t="n">
+        <v>3.0</v>
       </c>
     </row>
     <row r="53" ht="20" customHeight="1">
@@ -19892,19 +20557,32 @@
       <c r="D53" s="6" t="n">
         <v>18734.46</v>
       </c>
-      <c r="E53" s="6" t="n">
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>00035270</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>2024-12-04</t>
+        </is>
+      </c>
+      <c r="G53" s="6" t="n">
         <v>18441.12</v>
       </c>
-      <c r="F53" s="6" t="n">
+      <c r="H53" s="6" t="n">
+        <v>18441.12</v>
+      </c>
+      <c r="I53" s="6" t="n">
         <v>293.34</v>
       </c>
-      <c r="G53" s="5" t="inlineStr">
+      <c r="J53" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="H53" s="6" t="n">
-        <v>7</v>
+      <c r="K53" s="6" t="n">
+        <v>7.0</v>
       </c>
     </row>
     <row r="54" ht="20" customHeight="1">
@@ -19924,19 +20602,32 @@
       <c r="D54" s="6" t="n">
         <v>11105.31</v>
       </c>
-      <c r="E54" s="6" t="n">
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>00030891</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>2024-05-27</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="n">
         <v>11105.31</v>
       </c>
-      <c r="F54" s="6" t="n">
+      <c r="H54" s="6" t="n">
+        <v>11105.31</v>
+      </c>
+      <c r="I54" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G54" s="5" t="inlineStr">
+      <c r="J54" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H54" s="6" t="n">
-        <v>6</v>
+      <c r="K54" s="6" t="n">
+        <v>6.0</v>
       </c>
     </row>
     <row r="55" ht="20" customHeight="1">
@@ -19956,19 +20647,32 @@
       <c r="D55" s="6" t="n">
         <v>13862.53</v>
       </c>
-      <c r="E55" s="6" t="n">
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>00032896</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>2024-08-23</t>
+        </is>
+      </c>
+      <c r="G55" s="6" t="n">
+        <v>17634.86</v>
+      </c>
+      <c r="H55" s="6" t="n">
         <v>13862.53</v>
       </c>
-      <c r="F55" s="6" t="n">
+      <c r="I55" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G55" s="5" t="inlineStr">
+      <c r="J55" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H55" s="6" t="n">
-        <v>4</v>
+      <c r="K55" s="6" t="n">
+        <v>4.0</v>
       </c>
     </row>
     <row r="56" ht="20" customHeight="1">
@@ -19988,19 +20692,32 @@
       <c r="D56" s="6" t="n">
         <v>15395.18</v>
       </c>
-      <c r="E56" s="6" t="n">
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>00031792</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>2024-07-09</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="n">
         <v>15395.18</v>
       </c>
-      <c r="F56" s="6" t="n">
+      <c r="H56" s="6" t="n">
+        <v>15395.18</v>
+      </c>
+      <c r="I56" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G56" s="5" t="inlineStr">
+      <c r="J56" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H56" s="6" t="n">
-        <v>5</v>
+      <c r="K56" s="6" t="n">
+        <v>5.0</v>
       </c>
     </row>
     <row r="57" ht="20" customHeight="1">
@@ -20020,19 +20737,32 @@
       <c r="D57" s="6" t="n">
         <v>12634.86</v>
       </c>
-      <c r="E57" s="6" t="n">
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>00033810</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>2024-09-30</t>
+        </is>
+      </c>
+      <c r="G57" s="6" t="n">
+        <v>20232.18</v>
+      </c>
+      <c r="H57" s="6" t="n">
         <v>12634.86</v>
       </c>
-      <c r="F57" s="6" t="n">
+      <c r="I57" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G57" s="5" t="inlineStr">
+      <c r="J57" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H57" s="6" t="n">
-        <v>4</v>
+      <c r="K57" s="6" t="n">
+        <v>4.0</v>
       </c>
     </row>
     <row r="58" ht="20" customHeight="1">
@@ -20052,19 +20782,32 @@
       <c r="D58" s="6" t="n">
         <v>18256.94</v>
       </c>
-      <c r="E58" s="6" t="n">
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>00031179</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>2024-06-10</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="n">
         <v>13862.03</v>
       </c>
-      <c r="F58" s="6" t="n">
+      <c r="H58" s="6" t="n">
+        <v>13862.03</v>
+      </c>
+      <c r="I58" s="6" t="n">
         <v>4394.91</v>
       </c>
-      <c r="G58" s="5" t="inlineStr">
+      <c r="J58" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="H58" s="6" t="n">
-        <v>6</v>
+      <c r="K58" s="6" t="n">
+        <v>6.0</v>
       </c>
     </row>
     <row r="59" ht="20" customHeight="1">
@@ -20084,19 +20827,32 @@
       <c r="D59" s="6" t="n">
         <v>15232.18</v>
       </c>
-      <c r="E59" s="6" t="n">
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>00034425</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>2024-10-28</t>
+        </is>
+      </c>
+      <c r="G59" s="6" t="n">
+        <v>20443.0</v>
+      </c>
+      <c r="H59" s="6" t="n">
         <v>15232.18</v>
       </c>
-      <c r="F59" s="6" t="n">
+      <c r="I59" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G59" s="5" t="inlineStr">
+      <c r="J59" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H59" s="6" t="n">
-        <v>4</v>
+      <c r="K59" s="6" t="n">
+        <v>4.0</v>
       </c>
     </row>
     <row r="60" ht="20" customHeight="1">
@@ -20116,19 +20872,32 @@
       <c r="D60" s="6" t="n">
         <v>15443.0</v>
       </c>
-      <c r="E60" s="6" t="n">
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>00036139</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>2025-01-17</t>
+        </is>
+      </c>
+      <c r="G60" s="6" t="n">
+        <v>22336.89</v>
+      </c>
+      <c r="H60" s="6" t="n">
         <v>15443.0</v>
       </c>
-      <c r="F60" s="6" t="n">
+      <c r="I60" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G60" s="5" t="inlineStr">
+      <c r="J60" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H60" s="6" t="n">
-        <v>5</v>
+      <c r="K60" s="6" t="n">
+        <v>5.0</v>
       </c>
     </row>
     <row r="61" ht="20" customHeight="1">
@@ -20148,19 +20917,32 @@
       <c r="D61" s="6" t="n">
         <v>15184.18</v>
       </c>
-      <c r="E61" s="6" t="n">
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>00036988</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>2025-02-21</t>
+        </is>
+      </c>
+      <c r="G61" s="6" t="n">
+        <v>19550.42</v>
+      </c>
+      <c r="H61" s="6" t="n">
         <v>15184.18</v>
       </c>
-      <c r="F61" s="6" t="n">
+      <c r="I61" s="6" t="n">
         <v>-0.0</v>
       </c>
-      <c r="G61" s="5" t="inlineStr">
+      <c r="J61" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H61" s="6" t="n">
-        <v>5</v>
+      <c r="K61" s="6" t="n">
+        <v>5.0</v>
       </c>
     </row>
     <row r="62" ht="20" customHeight="1">
@@ -20180,19 +20962,34 @@
       <c r="D62" s="6" t="n">
         <v>15336.89</v>
       </c>
-      <c r="E62" s="6" t="n">
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="F62" s="6" t="n">
+      <c r="I62" s="6" t="n">
         <v>15336.89</v>
       </c>
-      <c r="G62" s="5" t="inlineStr">
+      <c r="J62" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="H62" s="6" t="n">
-        <v>5</v>
+      <c r="K62" s="6" t="n">
+        <v>5.0</v>
       </c>
     </row>
     <row r="63" ht="20" customHeight="1">
@@ -20212,19 +21009,34 @@
       <c r="D63" s="6" t="n">
         <v>14025.58</v>
       </c>
-      <c r="E63" s="6" t="n">
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="F63" s="6" t="n">
+      <c r="I63" s="6" t="n">
         <v>14025.58</v>
       </c>
-      <c r="G63" s="5" t="inlineStr">
+      <c r="J63" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="H63" s="6" t="n">
-        <v>7</v>
+      <c r="K63" s="6" t="n">
+        <v>7.0</v>
       </c>
     </row>
     <row r="64" ht="20" customHeight="1">
@@ -20244,19 +21056,34 @@
       <c r="D64" s="6" t="n">
         <v>12524.85</v>
       </c>
-      <c r="E64" s="6" t="n">
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="F64" s="6" t="n">
+      <c r="I64" s="6" t="n">
         <v>12524.85</v>
       </c>
-      <c r="G64" s="5" t="inlineStr">
+      <c r="J64" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="H64" s="6" t="n">
-        <v>4</v>
+      <c r="K64" s="6" t="n">
+        <v>4.0</v>
       </c>
     </row>
     <row r="65" ht="20" customHeight="1">
@@ -20276,19 +21103,32 @@
       <c r="D65" s="6" t="n">
         <v>15816.63</v>
       </c>
-      <c r="E65" s="6" t="n">
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>00038481</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>2025-05-05</t>
+        </is>
+      </c>
+      <c r="G65" s="6" t="n">
         <v>15816.63</v>
       </c>
-      <c r="F65" s="6" t="n">
+      <c r="H65" s="6" t="n">
+        <v>15816.63</v>
+      </c>
+      <c r="I65" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G65" s="5" t="inlineStr">
+      <c r="J65" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H65" s="6" t="n">
-        <v>4</v>
+      <c r="K65" s="6" t="n">
+        <v>4.0</v>
       </c>
     </row>
     <row r="66" ht="20" customHeight="1">
@@ -20308,19 +21148,34 @@
       <c r="D66" s="6" t="n">
         <v>17574.84</v>
       </c>
-      <c r="E66" s="6" t="n">
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="F66" s="6" t="n">
+      <c r="I66" s="6" t="n">
         <v>17574.84</v>
       </c>
-      <c r="G66" s="5" t="inlineStr">
+      <c r="J66" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="H66" s="6" t="n">
-        <v>5</v>
+      <c r="K66" s="6" t="n">
+        <v>5.0</v>
       </c>
     </row>
     <row r="67" ht="20" customHeight="1">
@@ -20340,19 +21195,34 @@
       <c r="D67" s="6" t="n">
         <v>10320.82</v>
       </c>
-      <c r="E67" s="6" t="n">
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="F67" s="6" t="n">
+      <c r="I67" s="6" t="n">
         <v>10320.82</v>
       </c>
-      <c r="G67" s="5" t="inlineStr">
+      <c r="J67" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="H67" s="6" t="n">
-        <v>3</v>
+      <c r="K67" s="6" t="n">
+        <v>3.0</v>
       </c>
     </row>
     <row r="68" ht="20" customHeight="1">
@@ -20372,19 +21242,32 @@
       <c r="D68" s="6" t="n">
         <v>11795.24</v>
       </c>
-      <c r="E68" s="6" t="n">
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>00040063</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>2025-07-14</t>
+        </is>
+      </c>
+      <c r="G68" s="6" t="n">
         <v>11795.24</v>
       </c>
-      <c r="F68" s="6" t="n">
+      <c r="H68" s="6" t="n">
+        <v>11795.24</v>
+      </c>
+      <c r="I68" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G68" s="5" t="inlineStr">
+      <c r="J68" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H68" s="6" t="n">
-        <v>4</v>
+      <c r="K68" s="6" t="n">
+        <v>4.0</v>
       </c>
     </row>
     <row r="69" ht="20" customHeight="1">
@@ -20404,19 +21287,34 @@
       <c r="D69" s="6" t="n">
         <v>21724.53</v>
       </c>
-      <c r="E69" s="6" t="n">
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="F69" s="6" t="n">
+      <c r="I69" s="6" t="n">
         <v>21724.53</v>
       </c>
-      <c r="G69" s="5" t="inlineStr">
+      <c r="J69" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="H69" s="6" t="n">
-        <v>5</v>
+      <c r="K69" s="6" t="n">
+        <v>5.0</v>
       </c>
     </row>
     <row r="70" ht="20" customHeight="1">
@@ -20436,19 +21334,34 @@
       <c r="D70" s="6" t="n">
         <v>13342.37</v>
       </c>
-      <c r="E70" s="6" t="n">
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H70" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="F70" s="6" t="n">
+      <c r="I70" s="6" t="n">
         <v>13342.37</v>
       </c>
-      <c r="G70" s="5" t="inlineStr">
+      <c r="J70" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="H70" s="6" t="n">
-        <v>6</v>
+      <c r="K70" s="6" t="n">
+        <v>6.0</v>
       </c>
     </row>
     <row r="71" ht="20" customHeight="1">
@@ -20468,19 +21381,32 @@
       <c r="D71" s="6" t="n">
         <v>14618.11</v>
       </c>
-      <c r="E71" s="6" t="n">
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>00040746</t>
+        </is>
+      </c>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>2025-08-22</t>
+        </is>
+      </c>
+      <c r="G71" s="6" t="n">
         <v>14579.44</v>
       </c>
-      <c r="F71" s="6" t="n">
+      <c r="H71" s="6" t="n">
+        <v>14579.44</v>
+      </c>
+      <c r="I71" s="6" t="n">
         <v>38.67</v>
       </c>
-      <c r="G71" s="5" t="inlineStr">
+      <c r="J71" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="H71" s="6" t="n">
-        <v>6</v>
+      <c r="K71" s="6" t="n">
+        <v>6.0</v>
       </c>
     </row>
     <row r="72" ht="20" customHeight="1">
@@ -20500,19 +21426,34 @@
       <c r="D72" s="6" t="n">
         <v>14579.44</v>
       </c>
-      <c r="E72" s="6" t="n">
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H72" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="F72" s="6" t="n">
+      <c r="I72" s="6" t="n">
         <v>14579.44</v>
       </c>
-      <c r="G72" s="5" t="inlineStr">
+      <c r="J72" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="H72" s="6" t="n">
-        <v>5</v>
+      <c r="K72" s="6" t="n">
+        <v>5.0</v>
       </c>
     </row>
     <row r="73" ht="20" customHeight="1">
@@ -20532,19 +21473,32 @@
       <c r="D73" s="6" t="n">
         <v>16601.82</v>
       </c>
-      <c r="E73" s="6" t="n">
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>00041664</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>2025-10-14</t>
+        </is>
+      </c>
+      <c r="G73" s="6" t="n">
         <v>16601.81</v>
       </c>
-      <c r="F73" s="6" t="n">
+      <c r="H73" s="6" t="n">
+        <v>16601.81</v>
+      </c>
+      <c r="I73" s="6" t="n">
         <v>0.01</v>
       </c>
-      <c r="G73" s="5" t="inlineStr">
+      <c r="J73" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H73" s="6" t="n">
-        <v>5</v>
+      <c r="K73" s="6" t="n">
+        <v>5.0</v>
       </c>
     </row>
     <row r="74" ht="20" customHeight="1">
@@ -20564,19 +21518,32 @@
       <c r="D74" s="6" t="n">
         <v>13327.87</v>
       </c>
-      <c r="E74" s="6" t="n">
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>00042134</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="G74" s="6" t="n">
         <v>13327.87</v>
       </c>
-      <c r="F74" s="6" t="n">
+      <c r="H74" s="6" t="n">
+        <v>13327.87</v>
+      </c>
+      <c r="I74" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G74" s="5" t="inlineStr">
+      <c r="J74" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H74" s="6" t="n">
-        <v>4</v>
+      <c r="K74" s="6" t="n">
+        <v>4.0</v>
       </c>
     </row>
     <row r="75" ht="20" customHeight="1">
@@ -20596,19 +21563,32 @@
       <c r="D75" s="6" t="n">
         <v>13161.86</v>
       </c>
-      <c r="E75" s="6" t="n">
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>00042788</t>
+        </is>
+      </c>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>2025-12-29</t>
+        </is>
+      </c>
+      <c r="G75" s="6" t="n">
         <v>13161.86</v>
       </c>
-      <c r="F75" s="6" t="n">
+      <c r="H75" s="6" t="n">
+        <v>13161.86</v>
+      </c>
+      <c r="I75" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G75" s="5" t="inlineStr">
+      <c r="J75" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H75" s="6" t="n">
-        <v>4</v>
+      <c r="K75" s="6" t="n">
+        <v>4.0</v>
       </c>
     </row>
     <row r="76" ht="20" customHeight="1">
@@ -20628,19 +21608,32 @@
       <c r="D76" s="6" t="n">
         <v>15578.23</v>
       </c>
-      <c r="E76" s="6" t="n">
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>00043199</t>
+        </is>
+      </c>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="G76" s="6" t="n">
         <v>15578.23</v>
       </c>
-      <c r="F76" s="6" t="n">
+      <c r="H76" s="6" t="n">
+        <v>15578.23</v>
+      </c>
+      <c r="I76" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="G76" s="5" t="inlineStr">
+      <c r="J76" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="H76" s="6" t="n">
-        <v>5</v>
+      <c r="K76" s="6" t="n">
+        <v>5.0</v>
       </c>
     </row>
     <row r="77" ht="20" customHeight="1">
@@ -20660,19 +21653,34 @@
       <c r="D77" s="6" t="n">
         <v>11666.11</v>
       </c>
-      <c r="E77" s="6" t="n">
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H77" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="F77" s="6" t="n">
+      <c r="I77" s="6" t="n">
         <v>11666.11</v>
       </c>
-      <c r="G77" s="5" t="inlineStr">
+      <c r="J77" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="H77" s="6" t="n">
-        <v>6</v>
+      <c r="K77" s="6" t="n">
+        <v>6.0</v>
       </c>
     </row>
     <row r="78" ht="20" customHeight="1">
@@ -20692,19 +21700,34 @@
       <c r="D78" s="6" t="n">
         <v>14323.09</v>
       </c>
-      <c r="E78" s="6" t="n">
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H78" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="F78" s="6" t="n">
+      <c r="I78" s="6" t="n">
         <v>14323.09</v>
       </c>
-      <c r="G78" s="5" t="inlineStr">
+      <c r="J78" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="H78" s="6" t="n">
-        <v>6</v>
+      <c r="K78" s="6" t="n">
+        <v>6.0</v>
       </c>
     </row>
     <row r="79" ht="20" customHeight="1">
@@ -20724,19 +21747,34 @@
       <c r="D79" s="6" t="n">
         <v>10559.95</v>
       </c>
-      <c r="E79" s="6" t="n">
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H79" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="F79" s="6" t="n">
+      <c r="I79" s="6" t="n">
         <v>10559.95</v>
       </c>
-      <c r="G79" s="5" t="inlineStr">
+      <c r="J79" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="H79" s="6" t="n">
-        <v>3</v>
+      <c r="K79" s="6" t="n">
+        <v>3.0</v>
       </c>
     </row>
     <row r="80" ht="20" customHeight="1">
@@ -20756,19 +21794,32 @@
       <c r="D80" s="6" t="n">
         <v>11937.56</v>
       </c>
-      <c r="E80" s="6" t="n">
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>00044555</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="G80" s="6" t="n">
         <v>11666.12</v>
       </c>
-      <c r="F80" s="6" t="n">
+      <c r="H80" s="6" t="n">
+        <v>11666.12</v>
+      </c>
+      <c r="I80" s="6" t="n">
         <v>271.44</v>
       </c>
-      <c r="G80" s="5" t="inlineStr">
+      <c r="J80" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="H80" s="6" t="n">
-        <v>5</v>
+      <c r="K80" s="6" t="n">
+        <v>5.0</v>
       </c>
     </row>
     <row r="81" ht="20" customHeight="1">
@@ -20788,19 +21839,34 @@
       <c r="D81" s="6" t="n">
         <v>14303.99</v>
       </c>
-      <c r="E81" s="6" t="n">
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H81" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="F81" s="6" t="n">
+      <c r="I81" s="6" t="n">
         <v>14303.99</v>
       </c>
-      <c r="G81" s="5" t="inlineStr">
+      <c r="J81" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="H81" s="6" t="n">
-        <v>4</v>
+      <c r="K81" s="6" t="n">
+        <v>4.0</v>
       </c>
     </row>
     <row r="82" ht="20" customHeight="1">
@@ -20820,23 +21886,38 @@
       <c r="D82" s="6" t="n">
         <v>21274.86</v>
       </c>
-      <c r="E82" s="6" t="n">
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H82" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="F82" s="6" t="n">
+      <c r="I82" s="6" t="n">
         <v>21274.86</v>
       </c>
-      <c r="G82" s="5" t="inlineStr">
+      <c r="J82" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="H82" s="6" t="n">
-        <v>5</v>
+      <c r="K82" s="6" t="n">
+        <v>5.0</v>
       </c>
     </row>
     <row r="83" ht="20" customHeight="1">
-      <c r="A83" s="2" t="inlineStr">
+      <c r="A83" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -20854,18 +21935,33 @@
       <c r="D83" s="6" t="n">
         <v>1102643.55</v>
       </c>
-      <c r="E83" s="6" t="n">
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H83" s="6" t="n">
         <v>836374.12</v>
       </c>
-      <c r="F83" s="6" t="n">
+      <c r="I83" s="6" t="n">
         <v>273153.18</v>
       </c>
-      <c r="G83" s="5" t="inlineStr">
+      <c r="J83" s="5" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="H83" s="5" t="inlineStr">
+      <c r="K83" s="5" t="inlineStr">
         <is>
           <t/>
         </is>

</xml_diff>

<commit_message>
JIM001 v4.1: add net invoiced less payment gross column on open-by-month sheet.
Derived monthly variance between LPG net and consolidated payment gross; regenerate workbook.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/analysis/debtors/JIM001/reports/JIM001_LPG_Reconciliation_v4.1.xlsx
+++ b/analysis/debtors/JIM001/reports/JIM001_LPG_Reconciliation_v4.1.xlsx
@@ -220,6 +220,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Claude (JIM001 bridge review)</author>
+  </authors>
+  <commentList>
+    <comment ref="B80" authorId="0" shapeId="0">
+      <text>
+        <t>Month attribution: December 2025 (aggregate exact-sum match, R0.01 variance -- rounding). ERP-ledger invoice-level split points to March 2026 instead but is unconfirmed (mechanical FIFO fill of an assumed month, same pattern as doc 40746's June/July case). ASSERTED, not PROVEN -- no remittance advice exists for JIM001. See JIM001_Exact_Sum_Bridge_Review_2026-09-13.md SS5.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Claude (JIM001 bridge review)</author>
+  </authors>
+  <commentList>
+    <comment ref="D30" authorId="0" shapeId="0">
+      <text>
+        <t>R0.01 variance (11,666.12 vs 11,666.11), same rounding tolerance treated as exact elsewhere in this sheet (e.g. docs 8420, 41664). ASSERTED via aggregate exact-sum match, not PROVEN -- no remittance advice exists for JIM001. Contradicts the unconfirmed ERP-ledger invoice split (allocation_edges.csv AL-0359-AL-0361) which points to March 2026 instead. See JIM001_Exact_Sum_Bridge_Review_2026-09-13.md SS5.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -573,9 +603,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr"/>
       <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E4" s="6" t="n"/>
       <c r="F4" s="6" t="n">
         <v>0</v>
       </c>
@@ -723,9 +751,7 @@
       </c>
       <c r="C11" s="8" t="inlineStr"/>
       <c r="D11" s="9" t="inlineStr"/>
-      <c r="E11" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E11" s="10" t="n"/>
       <c r="F11" s="10" t="n">
         <v>9000.02</v>
       </c>
@@ -1247,9 +1273,7 @@
       </c>
       <c r="C35" s="8" t="inlineStr"/>
       <c r="D35" s="9" t="inlineStr"/>
-      <c r="E35" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E35" s="10" t="n"/>
       <c r="F35" s="10" t="n">
         <v>11406.77</v>
       </c>
@@ -1595,9 +1619,7 @@
       </c>
       <c r="C51" s="8" t="inlineStr"/>
       <c r="D51" s="9" t="inlineStr"/>
-      <c r="E51" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E51" s="10" t="n"/>
       <c r="F51" s="10" t="n">
         <v>9756.790000000001</v>
       </c>
@@ -1899,9 +1921,7 @@
       </c>
       <c r="C65" s="8" t="inlineStr"/>
       <c r="D65" s="9" t="inlineStr"/>
-      <c r="E65" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E65" s="10" t="n"/>
       <c r="F65" s="10" t="n">
         <v>13531.77</v>
       </c>
@@ -2137,9 +2157,7 @@
       </c>
       <c r="C76" s="4" t="inlineStr"/>
       <c r="D76" s="5" t="inlineStr"/>
-      <c r="E76" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E76" s="6" t="n"/>
       <c r="F76" s="6" t="n">
         <v>17111.63</v>
       </c>
@@ -2331,9 +2349,7 @@
       </c>
       <c r="C85" s="8" t="inlineStr"/>
       <c r="D85" s="9" t="inlineStr"/>
-      <c r="E85" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E85" s="10" t="n"/>
       <c r="F85" s="10" t="n">
         <v>13817.26</v>
       </c>
@@ -2547,9 +2563,7 @@
       </c>
       <c r="C95" s="8" t="inlineStr"/>
       <c r="D95" s="9" t="inlineStr"/>
-      <c r="E95" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E95" s="10" t="n"/>
       <c r="F95" s="10" t="n">
         <v>16442.26</v>
       </c>
@@ -2851,9 +2865,7 @@
       </c>
       <c r="C109" s="8" t="inlineStr"/>
       <c r="D109" s="9" t="inlineStr"/>
-      <c r="E109" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E109" s="10" t="n"/>
       <c r="F109" s="10" t="n">
         <v>15673.27</v>
       </c>
@@ -3111,9 +3123,7 @@
       </c>
       <c r="C121" s="8" t="inlineStr"/>
       <c r="D121" s="9" t="inlineStr"/>
-      <c r="E121" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E121" s="10" t="n"/>
       <c r="F121" s="10" t="n">
         <v>15119.26</v>
       </c>
@@ -3349,9 +3359,7 @@
       </c>
       <c r="C132" s="4" t="inlineStr"/>
       <c r="D132" s="5" t="inlineStr"/>
-      <c r="E132" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E132" s="6" t="n"/>
       <c r="F132" s="6" t="n">
         <v>14567.24</v>
       </c>
@@ -3565,9 +3573,7 @@
       </c>
       <c r="C142" s="4" t="inlineStr"/>
       <c r="D142" s="5" t="inlineStr"/>
-      <c r="E142" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E142" s="6" t="n"/>
       <c r="F142" s="6" t="n">
         <v>13442.19</v>
       </c>
@@ -3803,9 +3809,7 @@
       </c>
       <c r="C153" s="8" t="inlineStr"/>
       <c r="D153" s="9" t="inlineStr"/>
-      <c r="E153" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E153" s="10" t="n"/>
       <c r="F153" s="10" t="n">
         <v>24482.13</v>
       </c>
@@ -4085,9 +4089,7 @@
       </c>
       <c r="C166" s="4" t="inlineStr"/>
       <c r="D166" s="5" t="inlineStr"/>
-      <c r="E166" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E166" s="6" t="n"/>
       <c r="F166" s="6" t="n">
         <v>13955.98</v>
       </c>
@@ -4323,9 +4325,7 @@
       </c>
       <c r="C177" s="8" t="inlineStr"/>
       <c r="D177" s="9" t="inlineStr"/>
-      <c r="E177" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E177" s="10" t="n"/>
       <c r="F177" s="10" t="n">
         <v>15081.07</v>
       </c>
@@ -4517,9 +4517,7 @@
       </c>
       <c r="C186" s="4" t="inlineStr"/>
       <c r="D186" s="5" t="inlineStr"/>
-      <c r="E186" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E186" s="6" t="n"/>
       <c r="F186" s="6" t="n">
         <v>26331.1</v>
       </c>
@@ -4711,9 +4709,7 @@
       </c>
       <c r="C195" s="8" t="inlineStr"/>
       <c r="D195" s="9" t="inlineStr"/>
-      <c r="E195" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E195" s="10" t="n"/>
       <c r="F195" s="10" t="n">
         <v>21153.33</v>
       </c>
@@ -4773,9 +4769,7 @@
       </c>
       <c r="C198" s="4" t="inlineStr"/>
       <c r="D198" s="5" t="inlineStr"/>
-      <c r="E198" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E198" s="6" t="n"/>
       <c r="F198" s="6" t="n">
         <v>12903.33</v>
       </c>
@@ -4813,9 +4807,7 @@
       </c>
       <c r="C200" s="4" t="inlineStr"/>
       <c r="D200" s="5" t="inlineStr"/>
-      <c r="E200" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E200" s="6" t="n"/>
       <c r="F200" s="6" t="n">
         <v>9903.33</v>
       </c>
@@ -4853,9 +4845,7 @@
       </c>
       <c r="C202" s="4" t="inlineStr"/>
       <c r="D202" s="5" t="inlineStr"/>
-      <c r="E202" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E202" s="6" t="n"/>
       <c r="F202" s="6" t="n">
         <v>4903.33</v>
       </c>
@@ -4893,9 +4883,7 @@
       </c>
       <c r="C204" s="4" t="inlineStr"/>
       <c r="D204" s="5" t="inlineStr"/>
-      <c r="E204" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E204" s="6" t="n"/>
       <c r="F204" s="6" t="n">
         <v>-221.67</v>
       </c>
@@ -5065,9 +5053,7 @@
       </c>
       <c r="C212" s="4" t="inlineStr"/>
       <c r="D212" s="5" t="inlineStr"/>
-      <c r="E212" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E212" s="6" t="n"/>
       <c r="F212" s="6" t="n">
         <v>12296.53</v>
       </c>
@@ -5259,9 +5245,7 @@
       </c>
       <c r="C221" s="8" t="inlineStr"/>
       <c r="D221" s="9" t="inlineStr"/>
-      <c r="E221" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E221" s="10" t="n"/>
       <c r="F221" s="10" t="n">
         <v>9544.08</v>
       </c>
@@ -5497,9 +5481,7 @@
       </c>
       <c r="C232" s="4" t="inlineStr"/>
       <c r="D232" s="5" t="inlineStr"/>
-      <c r="E232" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E232" s="6" t="n"/>
       <c r="F232" s="6" t="n">
         <v>12001.22</v>
       </c>
@@ -5757,9 +5739,7 @@
       </c>
       <c r="C244" s="4" t="inlineStr"/>
       <c r="D244" s="5" t="inlineStr"/>
-      <c r="E244" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E244" s="6" t="n"/>
       <c r="F244" s="6" t="n">
         <v>858.3099999999999</v>
       </c>
@@ -5907,9 +5887,7 @@
       </c>
       <c r="C251" s="8" t="inlineStr"/>
       <c r="D251" s="9" t="inlineStr"/>
-      <c r="E251" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E251" s="10" t="n"/>
       <c r="F251" s="10" t="n">
         <v>8858.26</v>
       </c>
@@ -6255,9 +6233,7 @@
       </c>
       <c r="C267" s="8" t="inlineStr"/>
       <c r="D267" s="9" t="inlineStr"/>
-      <c r="E267" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E267" s="10" t="n"/>
       <c r="F267" s="10" t="n">
         <v>12790.83</v>
       </c>
@@ -6537,9 +6513,7 @@
       </c>
       <c r="C280" s="4" t="inlineStr"/>
       <c r="D280" s="5" t="inlineStr"/>
-      <c r="E280" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E280" s="6" t="n"/>
       <c r="F280" s="6" t="n">
         <v>13038.61</v>
       </c>
@@ -6819,9 +6793,7 @@
       </c>
       <c r="C293" s="8" t="inlineStr"/>
       <c r="D293" s="9" t="inlineStr"/>
-      <c r="E293" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E293" s="10" t="n"/>
       <c r="F293" s="10" t="n">
         <v>13107.95</v>
       </c>
@@ -7079,9 +7051,7 @@
       </c>
       <c r="C305" s="8" t="inlineStr"/>
       <c r="D305" s="9" t="inlineStr"/>
-      <c r="E305" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E305" s="10" t="n"/>
       <c r="F305" s="10" t="n">
         <v>16557.15</v>
       </c>
@@ -7251,9 +7221,7 @@
       </c>
       <c r="C313" s="8" t="inlineStr"/>
       <c r="D313" s="9" t="inlineStr"/>
-      <c r="E313" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E313" s="10" t="n"/>
       <c r="F313" s="10" t="n">
         <v>16796.63</v>
       </c>
@@ -7467,9 +7435,7 @@
       </c>
       <c r="C323" s="8" t="inlineStr"/>
       <c r="D323" s="9" t="inlineStr"/>
-      <c r="E323" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E323" s="10" t="n"/>
       <c r="F323" s="10" t="n">
         <v>16203.91</v>
       </c>
@@ -7639,9 +7605,7 @@
       </c>
       <c r="C331" s="8" t="inlineStr"/>
       <c r="D331" s="9" t="inlineStr"/>
-      <c r="E331" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E331" s="10" t="n"/>
       <c r="F331" s="10" t="n">
         <v>28709.91</v>
       </c>
@@ -7877,9 +7841,7 @@
       </c>
       <c r="C342" s="4" t="inlineStr"/>
       <c r="D342" s="5" t="inlineStr"/>
-      <c r="E342" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E342" s="6" t="n"/>
       <c r="F342" s="6" t="n">
         <v>30678.89</v>
       </c>
@@ -8071,9 +8033,7 @@
       </c>
       <c r="C351" s="8" t="inlineStr"/>
       <c r="D351" s="9" t="inlineStr"/>
-      <c r="E351" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E351" s="10" t="n"/>
       <c r="F351" s="10" t="n">
         <v>32906.45</v>
       </c>
@@ -8309,9 +8269,7 @@
       </c>
       <c r="C362" s="4" t="inlineStr"/>
       <c r="D362" s="5" t="inlineStr"/>
-      <c r="E362" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E362" s="6" t="n"/>
       <c r="F362" s="6" t="n">
         <v>33669.38</v>
       </c>
@@ -8503,9 +8461,7 @@
       </c>
       <c r="C371" s="8" t="inlineStr"/>
       <c r="D371" s="9" t="inlineStr"/>
-      <c r="E371" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E371" s="10" t="n"/>
       <c r="F371" s="10" t="n">
         <v>49773.14</v>
       </c>
@@ -8653,9 +8609,7 @@
       </c>
       <c r="C378" s="4" t="inlineStr"/>
       <c r="D378" s="5" t="inlineStr"/>
-      <c r="E378" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E378" s="6" t="n"/>
       <c r="F378" s="6" t="n">
         <v>49666.76</v>
       </c>
@@ -8913,9 +8867,7 @@
       </c>
       <c r="C390" s="4" t="inlineStr"/>
       <c r="D390" s="5" t="inlineStr"/>
-      <c r="E390" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E390" s="6" t="n"/>
       <c r="F390" s="6" t="n">
         <v>53282.99</v>
       </c>
@@ -9063,9 +9015,7 @@
       </c>
       <c r="C397" s="8" t="inlineStr"/>
       <c r="D397" s="9" t="inlineStr"/>
-      <c r="E397" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E397" s="10" t="n"/>
       <c r="F397" s="10" t="n">
         <v>52719.78</v>
       </c>
@@ -9191,9 +9141,7 @@
       </c>
       <c r="C403" s="8" t="inlineStr"/>
       <c r="D403" s="9" t="inlineStr"/>
-      <c r="E403" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E403" s="10" t="n"/>
       <c r="F403" s="10" t="n">
         <v>49289.07</v>
       </c>
@@ -9429,9 +9377,7 @@
       </c>
       <c r="C414" s="4" t="inlineStr"/>
       <c r="D414" s="5" t="inlineStr"/>
-      <c r="E414" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E414" s="6" t="n"/>
       <c r="F414" s="6" t="n">
         <v>49494.29</v>
       </c>
@@ -9623,9 +9569,7 @@
       </c>
       <c r="C423" s="8" t="inlineStr"/>
       <c r="D423" s="9" t="inlineStr"/>
-      <c r="E423" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E423" s="10" t="n"/>
       <c r="F423" s="10" t="n">
         <v>53471.03</v>
       </c>
@@ -9751,9 +9695,7 @@
       </c>
       <c r="C429" s="8" t="inlineStr"/>
       <c r="D429" s="9" t="inlineStr"/>
-      <c r="E429" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E429" s="10" t="n"/>
       <c r="F429" s="10" t="n">
         <v>53980.79</v>
       </c>
@@ -9857,9 +9799,7 @@
       </c>
       <c r="C434" s="4" t="inlineStr"/>
       <c r="D434" s="5" t="inlineStr"/>
-      <c r="E434" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E434" s="6" t="n"/>
       <c r="F434" s="6" t="n">
         <v>41139.5</v>
       </c>
@@ -9985,9 +9925,7 @@
       </c>
       <c r="C440" s="4" t="inlineStr"/>
       <c r="D440" s="5" t="inlineStr"/>
-      <c r="E440" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E440" s="6" t="n"/>
       <c r="F440" s="6" t="n">
         <v>45915.32</v>
       </c>
@@ -10091,9 +10029,7 @@
       </c>
       <c r="C445" s="8" t="inlineStr"/>
       <c r="D445" s="9" t="inlineStr"/>
-      <c r="E445" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E445" s="10" t="n"/>
       <c r="F445" s="10" t="n">
         <v>61056.01</v>
       </c>
@@ -10263,9 +10199,7 @@
       </c>
       <c r="C453" s="8" t="inlineStr"/>
       <c r="D453" s="9" t="inlineStr"/>
-      <c r="E453" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E453" s="10" t="n"/>
       <c r="F453" s="10" t="n">
         <v>50672.03</v>
       </c>
@@ -10369,9 +10303,7 @@
       </c>
       <c r="C458" s="4" t="inlineStr"/>
       <c r="D458" s="5" t="inlineStr"/>
-      <c r="E458" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E458" s="6" t="n"/>
       <c r="F458" s="6" t="n">
         <v>64075.09</v>
       </c>
@@ -10519,9 +10451,7 @@
       </c>
       <c r="C465" s="8" t="inlineStr"/>
       <c r="D465" s="9" t="inlineStr"/>
-      <c r="E465" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E465" s="10" t="n"/>
       <c r="F465" s="10" t="n">
         <v>62845.94</v>
       </c>
@@ -10691,9 +10621,7 @@
       </c>
       <c r="C473" s="8" t="inlineStr"/>
       <c r="D473" s="9" t="inlineStr"/>
-      <c r="E473" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E473" s="10" t="n"/>
       <c r="F473" s="10" t="n">
         <v>61559.98</v>
       </c>
@@ -10841,9 +10769,7 @@
       </c>
       <c r="C480" s="4" t="inlineStr"/>
       <c r="D480" s="5" t="inlineStr"/>
-      <c r="E480" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E480" s="6" t="n"/>
       <c r="F480" s="6" t="n">
         <v>55867.88</v>
       </c>
@@ -10991,9 +10917,7 @@
       </c>
       <c r="C487" s="8" t="inlineStr"/>
       <c r="D487" s="9" t="inlineStr"/>
-      <c r="E487" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E487" s="10" t="n"/>
       <c r="F487" s="10" t="n">
         <v>55484.88</v>
       </c>
@@ -11119,9 +11043,7 @@
       </c>
       <c r="C493" s="8" t="inlineStr"/>
       <c r="D493" s="9" t="inlineStr"/>
-      <c r="E493" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E493" s="10" t="n"/>
       <c r="F493" s="10" t="n">
         <v>57172.55</v>
       </c>
@@ -11291,9 +11213,7 @@
       </c>
       <c r="C501" s="8" t="inlineStr"/>
       <c r="D501" s="9" t="inlineStr"/>
-      <c r="E501" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E501" s="10" t="n"/>
       <c r="F501" s="10" t="n">
         <v>48522.37</v>
       </c>
@@ -11463,9 +11383,7 @@
       </c>
       <c r="C509" s="8" t="inlineStr"/>
       <c r="D509" s="9" t="inlineStr"/>
-      <c r="E509" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E509" s="10" t="n"/>
       <c r="F509" s="10" t="n">
         <v>63749.15</v>
       </c>
@@ -11591,9 +11509,7 @@
       </c>
       <c r="C515" s="8" t="inlineStr"/>
       <c r="D515" s="9" t="inlineStr"/>
-      <c r="E515" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E515" s="10" t="n"/>
       <c r="F515" s="10" t="n">
         <v>62064.78</v>
       </c>
@@ -11697,9 +11613,7 @@
       </c>
       <c r="C520" s="4" t="inlineStr"/>
       <c r="D520" s="5" t="inlineStr"/>
-      <c r="E520" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E520" s="6" t="n"/>
       <c r="F520" s="6" t="n">
         <v>74676.91</v>
       </c>
@@ -11825,9 +11739,7 @@
       </c>
       <c r="C526" s="4" t="inlineStr"/>
       <c r="D526" s="5" t="inlineStr"/>
-      <c r="E526" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E526" s="6" t="n"/>
       <c r="F526" s="6" t="n">
         <v>71160.73</v>
       </c>
@@ -11997,9 +11909,7 @@
       </c>
       <c r="C534" s="4" t="inlineStr"/>
       <c r="D534" s="5" t="inlineStr"/>
-      <c r="E534" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E534" s="6" t="n"/>
       <c r="F534" s="6" t="n">
         <v>78312.36</v>
       </c>
@@ -12125,9 +12035,7 @@
       </c>
       <c r="C540" s="4" t="inlineStr"/>
       <c r="D540" s="5" t="inlineStr"/>
-      <c r="E540" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E540" s="6" t="n"/>
       <c r="F540" s="6" t="n">
         <v>79682.50999999999</v>
       </c>
@@ -12319,9 +12227,7 @@
       </c>
       <c r="C549" s="8" t="inlineStr"/>
       <c r="D549" s="9" t="inlineStr"/>
-      <c r="E549" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E549" s="10" t="n"/>
       <c r="F549" s="10" t="n">
         <v>79730.33</v>
       </c>
@@ -12469,9 +12375,7 @@
       </c>
       <c r="C556" s="4" t="inlineStr"/>
       <c r="D556" s="5" t="inlineStr"/>
-      <c r="E556" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E556" s="6" t="n"/>
       <c r="F556" s="6" t="n">
         <v>77279.64999999999</v>
       </c>
@@ -12619,9 +12523,7 @@
       </c>
       <c r="C563" s="8" t="inlineStr"/>
       <c r="D563" s="9" t="inlineStr"/>
-      <c r="E563" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E563" s="10" t="n"/>
       <c r="F563" s="10" t="n">
         <v>72384.36</v>
       </c>
@@ -12813,9 +12715,7 @@
       </c>
       <c r="C572" s="4" t="inlineStr"/>
       <c r="D572" s="5" t="inlineStr"/>
-      <c r="E572" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E572" s="6" t="n"/>
       <c r="F572" s="6" t="n">
         <v>65966.94</v>
       </c>
@@ -12919,9 +12819,7 @@
       </c>
       <c r="C577" s="8" t="inlineStr"/>
       <c r="D577" s="9" t="inlineStr"/>
-      <c r="E577" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E577" s="10" t="n"/>
       <c r="F577" s="10" t="n">
         <v>78491.78999999999</v>
       </c>
@@ -13047,9 +12945,7 @@
       </c>
       <c r="C583" s="8" t="inlineStr"/>
       <c r="D583" s="9" t="inlineStr"/>
-      <c r="E583" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E583" s="10" t="n"/>
       <c r="F583" s="10" t="n">
         <v>75867.3</v>
       </c>
@@ -13197,9 +13093,7 @@
       </c>
       <c r="C590" s="4" t="inlineStr"/>
       <c r="D590" s="5" t="inlineStr"/>
-      <c r="E590" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E590" s="6" t="n"/>
       <c r="F590" s="6" t="n">
         <v>71105.25</v>
       </c>
@@ -13303,9 +13197,7 @@
       </c>
       <c r="C595" s="8" t="inlineStr"/>
       <c r="D595" s="9" t="inlineStr"/>
-      <c r="E595" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E595" s="10" t="n"/>
       <c r="F595" s="10" t="n">
         <v>61875.65</v>
       </c>
@@ -13409,9 +13301,7 @@
       </c>
       <c r="C600" s="4" t="inlineStr"/>
       <c r="D600" s="5" t="inlineStr"/>
-      <c r="E600" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E600" s="6" t="n"/>
       <c r="F600" s="6" t="n">
         <v>73670.89</v>
       </c>
@@ -13537,9 +13427,7 @@
       </c>
       <c r="C606" s="4" t="inlineStr"/>
       <c r="D606" s="5" t="inlineStr"/>
-      <c r="E606" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E606" s="6" t="n"/>
       <c r="F606" s="6" t="n">
         <v>95395.42</v>
       </c>
@@ -13731,9 +13619,7 @@
       </c>
       <c r="C615" s="8" t="inlineStr"/>
       <c r="D615" s="9" t="inlineStr"/>
-      <c r="E615" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E615" s="10" t="n"/>
       <c r="F615" s="10" t="n">
         <v>85583.19</v>
       </c>
@@ -13903,9 +13789,7 @@
       </c>
       <c r="C623" s="8" t="inlineStr"/>
       <c r="D623" s="9" t="inlineStr"/>
-      <c r="E623" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E623" s="10" t="n"/>
       <c r="F623" s="10" t="n">
         <v>79643.61</v>
       </c>
@@ -14075,9 +13959,7 @@
       </c>
       <c r="C631" s="8" t="inlineStr"/>
       <c r="D631" s="9" t="inlineStr"/>
-      <c r="E631" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E631" s="10" t="n"/>
       <c r="F631" s="10" t="n">
         <v>86628.5</v>
       </c>
@@ -14203,9 +14085,7 @@
       </c>
       <c r="C637" s="8" t="inlineStr"/>
       <c r="D637" s="9" t="inlineStr"/>
-      <c r="E637" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E637" s="10" t="n"/>
       <c r="F637" s="10" t="n">
         <v>84450.19</v>
       </c>
@@ -14309,9 +14189,7 @@
       </c>
       <c r="C642" s="4" t="inlineStr"/>
       <c r="D642" s="5" t="inlineStr"/>
-      <c r="E642" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E642" s="6" t="n"/>
       <c r="F642" s="6" t="n">
         <v>97778.06</v>
       </c>
@@ -14459,9 +14337,7 @@
       </c>
       <c r="C649" s="8" t="inlineStr"/>
       <c r="D649" s="9" t="inlineStr"/>
-      <c r="E649" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E649" s="10" t="n"/>
       <c r="F649" s="10" t="n">
         <v>98286.67</v>
       </c>
@@ -14587,9 +14463,7 @@
       </c>
       <c r="C655" s="8" t="inlineStr"/>
       <c r="D655" s="9" t="inlineStr"/>
-      <c r="E655" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E655" s="10" t="n"/>
       <c r="F655" s="10" t="n">
         <v>96588.47</v>
       </c>
@@ -14781,9 +14655,7 @@
       </c>
       <c r="C664" s="4" t="inlineStr"/>
       <c r="D664" s="5" t="inlineStr"/>
-      <c r="E664" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E664" s="6" t="n"/>
       <c r="F664" s="6" t="n">
         <v>98987.49000000001</v>
       </c>
@@ -14909,9 +14781,7 @@
       </c>
       <c r="C670" s="4" t="inlineStr"/>
       <c r="D670" s="5" t="inlineStr"/>
-      <c r="E670" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E670" s="6" t="n"/>
       <c r="F670" s="6" t="n">
         <v>109415.81</v>
       </c>
@@ -15015,9 +14885,7 @@
       </c>
       <c r="C675" s="8" t="inlineStr"/>
       <c r="D675" s="9" t="inlineStr"/>
-      <c r="E675" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E675" s="10" t="n"/>
       <c r="F675" s="10" t="n">
         <v>104397.53</v>
       </c>
@@ -15165,9 +15033,7 @@
       </c>
       <c r="C682" s="4" t="inlineStr"/>
       <c r="D682" s="5" t="inlineStr"/>
-      <c r="E682" s="6" t="n">
-        <v/>
-      </c>
+      <c r="E682" s="6" t="n"/>
       <c r="F682" s="6" t="n">
         <v>120323.88</v>
       </c>
@@ -15271,9 +15137,7 @@
       </c>
       <c r="C687" s="8" t="inlineStr"/>
       <c r="D687" s="9" t="inlineStr"/>
-      <c r="E687" s="10" t="n">
-        <v/>
-      </c>
+      <c r="E687" s="10" t="n"/>
       <c r="F687" s="10" t="n">
         <v>135059.88</v>
       </c>
@@ -15373,7 +15237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F80"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -17509,17 +17373,45 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="11" t="inlineStr">
+      <c r="A80" s="7" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B80" s="8" t="inlineStr">
+        <is>
+          <t>00044555</t>
+        </is>
+      </c>
+      <c r="C80" s="9" t="inlineStr">
+        <is>
+          <t>Alloc</t>
+        </is>
+      </c>
+      <c r="D80" s="9" t="inlineStr">
+        <is>
+          <t>TRANSF</t>
+        </is>
+      </c>
+      <c r="E80" s="8" t="inlineStr">
+        <is>
+          <t>STAT 127</t>
+        </is>
+      </c>
+      <c r="F80" s="10" t="n">
+        <v>-11666.12</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="11" t="inlineStr">
         <is>
           <t>Total Payments Received</t>
         </is>
       </c>
-      <c r="B80" s="12" t="n"/>
-      <c r="C80" s="12" t="n"/>
-      <c r="D80" s="12" t="n"/>
-      <c r="E80" s="12" t="n"/>
-      <c r="F80" s="13">
-        <f>SUM(F4:F79)</f>
+      <c r="B81" s="12" t="n"/>
+      <c r="C81" s="12" t="n"/>
+      <c r="D81" s="12" t="n"/>
+      <c r="E81" s="12" t="n"/>
+      <c r="F81" s="13">
+        <f>SUM(F4:F80)</f>
         <v/>
       </c>
     </row>
@@ -17528,6 +17420,7 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -17537,7 +17430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -18213,20 +18106,44 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="inlineStr">
+      <c r="A30" s="10" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="n">
+        <v>11666.11</v>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>00044555</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>46178</v>
+      </c>
+      <c r="F30" s="10" t="n">
+        <v>11666.12</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>Total Matched LPG Sales</t>
         </is>
       </c>
-      <c r="B30" s="12" t="n"/>
-      <c r="C30" s="13">
-        <f>SUM(C4:C29)</f>
+      <c r="B31" s="12" t="n"/>
+      <c r="C31" s="13">
+        <f>SUM(C4:C30)</f>
         <v/>
       </c>
-      <c r="D30" s="12" t="n"/>
-      <c r="E30" s="12" t="n"/>
-      <c r="F30" s="13">
-        <f>SUM(F4:F29)</f>
+      <c r="D31" s="12" t="n"/>
+      <c r="E31" s="12" t="n"/>
+      <c r="F31" s="13">
+        <f>SUM(F4:F30)</f>
         <v/>
       </c>
     </row>
@@ -18235,6 +18152,7 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -18244,7 +18162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K83"/>
+  <dimension ref="A1:L83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18254,10 +18172,11 @@
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -18306,20 +18225,25 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
+          <t>Net LPG Invoiced less Payment Gross (Original)</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
           <t>Payment Allocated (Month)</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Open Invoices (Sum)</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Month Status</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>LPG Invoice Doc Count</t>
         </is>
@@ -18356,17 +18280,20 @@
         <v>7000.0</v>
       </c>
       <c r="H4" s="6" t="n">
+        <v>2000.02</v>
+      </c>
+      <c r="I4" s="6" t="n">
         <v>6556.68</v>
       </c>
-      <c r="I4" s="6" t="n">
+      <c r="J4" s="6" t="n">
         <v>2443.34</v>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="K4" s="6" t="n">
+      <c r="L4" s="6" t="n">
         <v>2.0</v>
       </c>
     </row>
@@ -18402,18 +18329,23 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="I5" s="6" t="n">
+      <c r="J5" s="6" t="n">
         <v>19306.77</v>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="K5" s="6" t="n">
+      <c r="L5" s="6" t="n">
         <v>19.0</v>
       </c>
     </row>
@@ -18448,17 +18380,20 @@
         <v>9925.0</v>
       </c>
       <c r="H6" s="6" t="n">
+        <v>172.41</v>
+      </c>
+      <c r="I6" s="6" t="n">
         <v>9925.0</v>
       </c>
-      <c r="I6" s="6" t="n">
+      <c r="J6" s="6" t="n">
         <v>172.41</v>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="K6" s="6" t="n">
+      <c r="L6" s="6" t="n">
         <v>11.0</v>
       </c>
     </row>
@@ -18494,18 +18429,23 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="I7" s="6" t="n">
+      <c r="J7" s="6" t="n">
         <v>4374.98</v>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="K7" s="6" t="n">
+      <c r="L7" s="6" t="n">
         <v>14.0</v>
       </c>
     </row>
@@ -18540,17 +18480,20 @@
         <v>13505.0</v>
       </c>
       <c r="H8" s="6" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="I8" s="6" t="n">
         <v>13504.86</v>
       </c>
-      <c r="I8" s="6" t="n">
+      <c r="J8" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K8" s="6" t="n">
+      <c r="L8" s="6" t="n">
         <v>9.0</v>
       </c>
     </row>
@@ -18585,17 +18528,20 @@
         <v>8625.0</v>
       </c>
       <c r="H9" s="6" t="n">
+        <v>85.63</v>
+      </c>
+      <c r="I9" s="6" t="n">
         <v>8625.0</v>
       </c>
-      <c r="I9" s="6" t="n">
+      <c r="J9" s="6" t="n">
         <v>85.63</v>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="K9" s="6" t="n">
+      <c r="L9" s="6" t="n">
         <v>6.0</v>
       </c>
     </row>
@@ -18630,17 +18576,20 @@
         <v>12750.0</v>
       </c>
       <c r="H10" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I10" s="6" t="n">
         <v>12750.0</v>
       </c>
-      <c r="I10" s="6" t="n">
+      <c r="J10" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K10" s="6" t="n">
+      <c r="L10" s="6" t="n">
         <v>9.0</v>
       </c>
     </row>
@@ -18675,17 +18624,20 @@
         <v>14429.0</v>
       </c>
       <c r="H11" s="6" t="n">
+        <v>552.01</v>
+      </c>
+      <c r="I11" s="6" t="n">
         <v>14429.0</v>
       </c>
-      <c r="I11" s="6" t="n">
+      <c r="J11" s="6" t="n">
         <v>552.01</v>
       </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="K11" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="K11" s="6" t="n">
+      <c r="L11" s="6" t="n">
         <v>11.0</v>
       </c>
     </row>
@@ -18720,17 +18672,20 @@
         <v>13875.0</v>
       </c>
       <c r="H12" s="6" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="I12" s="6" t="n">
         <v>13874.99</v>
       </c>
-      <c r="I12" s="6" t="n">
+      <c r="J12" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K12" s="6" t="n">
+      <c r="L12" s="6" t="n">
         <v>10.0</v>
       </c>
     </row>
@@ -18765,17 +18720,20 @@
         <v>13875.0</v>
       </c>
       <c r="H13" s="6" t="n">
+        <v>-552.02</v>
+      </c>
+      <c r="I13" s="6" t="n">
         <v>13874.98</v>
       </c>
-      <c r="I13" s="6" t="n">
+      <c r="J13" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="K13" s="5" t="inlineStr">
         <is>
           <t>OVERPAID</t>
         </is>
       </c>
-      <c r="K13" s="6" t="n">
+      <c r="L13" s="6" t="n">
         <v>9.0</v>
       </c>
     </row>
@@ -18810,17 +18768,20 @@
         <v>10875.0</v>
       </c>
       <c r="H14" s="6" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="I14" s="6" t="n">
         <v>10874.96</v>
       </c>
-      <c r="I14" s="6" t="n">
+      <c r="J14" s="6" t="n">
         <v>-0.0</v>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K14" s="6" t="n">
+      <c r="L14" s="6" t="n">
         <v>7.0</v>
       </c>
     </row>
@@ -18855,17 +18816,20 @@
         <v>12915.0</v>
       </c>
       <c r="H15" s="6" t="n">
+        <v>-0.07</v>
+      </c>
+      <c r="I15" s="6" t="n">
         <v>12914.93</v>
       </c>
-      <c r="I15" s="6" t="n">
+      <c r="J15" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J15" s="5" t="inlineStr">
+      <c r="K15" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K15" s="6" t="n">
+      <c r="L15" s="6" t="n">
         <v>11.0</v>
       </c>
     </row>
@@ -18900,17 +18864,20 @@
         <v>12715.0</v>
       </c>
       <c r="H16" s="6" t="n">
+        <v>16.05</v>
+      </c>
+      <c r="I16" s="6" t="n">
         <v>12715.0</v>
       </c>
-      <c r="I16" s="6" t="n">
+      <c r="J16" s="6" t="n">
         <v>16.05</v>
       </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="K16" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="K16" s="6" t="n">
+      <c r="L16" s="6" t="n">
         <v>8.0</v>
       </c>
     </row>
@@ -18945,17 +18912,20 @@
         <v>15302.8</v>
       </c>
       <c r="H17" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="I17" s="6" t="n">
         <v>15302.8</v>
       </c>
-      <c r="I17" s="6" t="n">
+      <c r="J17" s="6" t="n">
         <v>0.09</v>
       </c>
-      <c r="J17" s="5" t="inlineStr">
+      <c r="K17" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="K17" s="6" t="n">
+      <c r="L17" s="6" t="n">
         <v>10.0</v>
       </c>
     </row>
@@ -18991,18 +18961,23 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H18" s="6" t="n">
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="I18" s="6" t="n">
+      <c r="J18" s="6" t="n">
         <v>11250.03</v>
       </c>
-      <c r="J18" s="5" t="inlineStr">
+      <c r="K18" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="K18" s="6" t="n">
+      <c r="L18" s="6" t="n">
         <v>8.0</v>
       </c>
     </row>
@@ -19038,18 +19013,23 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H19" s="6" t="n">
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="I19" s="6" t="n">
+      <c r="J19" s="6" t="n">
         <v>10125.03</v>
       </c>
-      <c r="J19" s="5" t="inlineStr">
+      <c r="K19" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="K19" s="6" t="n">
+      <c r="L19" s="6" t="n">
         <v>7.0</v>
       </c>
     </row>
@@ -19084,17 +19064,20 @@
         <v>12518.21</v>
       </c>
       <c r="H20" s="6" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="I20" s="6" t="n">
         <v>12518.2</v>
       </c>
-      <c r="I20" s="6" t="n">
+      <c r="J20" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J20" s="5" t="inlineStr">
+      <c r="K20" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K20" s="6" t="n">
+      <c r="L20" s="6" t="n">
         <v>7.0</v>
       </c>
     </row>
@@ -19129,17 +19112,20 @@
         <v>9765.76</v>
       </c>
       <c r="H21" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I21" s="6" t="n">
         <v>9765.76</v>
       </c>
-      <c r="I21" s="6" t="n">
+      <c r="J21" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J21" s="5" t="inlineStr">
+      <c r="K21" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K21" s="6" t="n">
+      <c r="L21" s="6" t="n">
         <v>7.0</v>
       </c>
     </row>
@@ -19174,17 +19160,20 @@
         <v>12222.9</v>
       </c>
       <c r="H22" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I22" s="6" t="n">
         <v>12222.9</v>
       </c>
-      <c r="I22" s="6" t="n">
+      <c r="J22" s="6" t="n">
         <v>-0.0</v>
       </c>
-      <c r="J22" s="5" t="inlineStr">
+      <c r="K22" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K22" s="6" t="n">
+      <c r="L22" s="6" t="n">
         <v>9.0</v>
       </c>
     </row>
@@ -19219,17 +19208,20 @@
         <v>11292.11</v>
       </c>
       <c r="H23" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I23" s="6" t="n">
         <v>11292.11</v>
       </c>
-      <c r="I23" s="6" t="n">
+      <c r="J23" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J23" s="5" t="inlineStr">
+      <c r="K23" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K23" s="6" t="n">
+      <c r="L23" s="6" t="n">
         <v>8.0</v>
       </c>
     </row>
@@ -19264,17 +19256,20 @@
         <v>9079.94</v>
       </c>
       <c r="H24" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I24" s="6" t="n">
         <v>9079.94</v>
       </c>
-      <c r="I24" s="6" t="n">
+      <c r="J24" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J24" s="5" t="inlineStr">
+      <c r="K24" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K24" s="6" t="n">
+      <c r="L24" s="6" t="n">
         <v>7.0</v>
       </c>
     </row>
@@ -19309,17 +19304,20 @@
         <v>13012.5</v>
       </c>
       <c r="H25" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I25" s="6" t="n">
         <v>13012.5</v>
       </c>
-      <c r="I25" s="6" t="n">
+      <c r="J25" s="6" t="n">
         <v>0.01</v>
       </c>
-      <c r="J25" s="5" t="inlineStr">
+      <c r="K25" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K25" s="6" t="n">
+      <c r="L25" s="6" t="n">
         <v>15.0</v>
       </c>
     </row>
@@ -19354,17 +19352,20 @@
         <v>13260.28</v>
       </c>
       <c r="H26" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I26" s="6" t="n">
         <v>13260.28</v>
       </c>
-      <c r="I26" s="6" t="n">
+      <c r="J26" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J26" s="5" t="inlineStr">
+      <c r="K26" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K26" s="6" t="n">
+      <c r="L26" s="6" t="n">
         <v>11.0</v>
       </c>
     </row>
@@ -19399,17 +19400,20 @@
         <v>12929.71</v>
       </c>
       <c r="H27" s="6" t="n">
+        <v>399.91</v>
+      </c>
+      <c r="I27" s="6" t="n">
         <v>12929.71</v>
       </c>
-      <c r="I27" s="6" t="n">
+      <c r="J27" s="6" t="n">
         <v>399.91</v>
       </c>
-      <c r="J27" s="5" t="inlineStr">
+      <c r="K27" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="K27" s="6" t="n">
+      <c r="L27" s="6" t="n">
         <v>11.0</v>
       </c>
     </row>
@@ -19444,17 +19448,20 @@
         <v>17018.3</v>
       </c>
       <c r="H28" s="6" t="n">
+        <v>-639.39</v>
+      </c>
+      <c r="I28" s="6" t="n">
         <v>16778.82</v>
       </c>
-      <c r="I28" s="6" t="n">
+      <c r="J28" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J28" s="5" t="inlineStr">
+      <c r="K28" s="5" t="inlineStr">
         <is>
           <t>OVERPAID</t>
         </is>
       </c>
-      <c r="K28" s="6" t="n">
+      <c r="L28" s="6" t="n">
         <v>10.0</v>
       </c>
     </row>
@@ -19489,17 +19496,20 @@
         <v>12160.3</v>
       </c>
       <c r="H29" s="6" t="n">
+        <v>239.48</v>
+      </c>
+      <c r="I29" s="6" t="n">
         <v>12160.3</v>
       </c>
-      <c r="I29" s="6" t="n">
+      <c r="J29" s="6" t="n">
         <v>239.48</v>
       </c>
-      <c r="J29" s="5" t="inlineStr">
+      <c r="K29" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="K29" s="6" t="n">
+      <c r="L29" s="6" t="n">
         <v>6.0</v>
       </c>
     </row>
@@ -19534,17 +19544,20 @@
         <v>14982.58</v>
       </c>
       <c r="H30" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I30" s="6" t="n">
         <v>14982.58</v>
       </c>
-      <c r="I30" s="6" t="n">
+      <c r="J30" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J30" s="5" t="inlineStr">
+      <c r="K30" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K30" s="6" t="n">
+      <c r="L30" s="6" t="n">
         <v>7.0</v>
       </c>
     </row>
@@ -19579,17 +19592,20 @@
         <v>13949.0</v>
       </c>
       <c r="H31" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I31" s="6" t="n">
         <v>13949.0</v>
       </c>
-      <c r="I31" s="6" t="n">
+      <c r="J31" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J31" s="5" t="inlineStr">
+      <c r="K31" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K31" s="6" t="n">
+      <c r="L31" s="6" t="n">
         <v>8.0</v>
       </c>
     </row>
@@ -19625,18 +19641,23 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H32" s="6" t="n">
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="I32" s="6" t="n">
+      <c r="J32" s="6" t="n">
         <v>14943.48</v>
       </c>
-      <c r="J32" s="5" t="inlineStr">
+      <c r="K32" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="K32" s="6" t="n">
+      <c r="L32" s="6" t="n">
         <v>8.0</v>
       </c>
     </row>
@@ -19671,17 +19692,20 @@
         <v>18184.64</v>
       </c>
       <c r="H33" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I33" s="6" t="n">
         <v>18184.64</v>
       </c>
-      <c r="I33" s="6" t="n">
+      <c r="J33" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J33" s="5" t="inlineStr">
+      <c r="K33" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K33" s="6" t="n">
+      <c r="L33" s="6" t="n">
         <v>8.0</v>
       </c>
     </row>
@@ -19716,17 +19740,20 @@
         <v>17275.67</v>
       </c>
       <c r="H34" s="6" t="n">
+        <v>1671.9</v>
+      </c>
+      <c r="I34" s="6" t="n">
         <v>17275.67</v>
       </c>
-      <c r="I34" s="6" t="n">
+      <c r="J34" s="6" t="n">
         <v>1671.9</v>
       </c>
-      <c r="J34" s="5" t="inlineStr">
+      <c r="K34" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="K34" s="6" t="n">
+      <c r="L34" s="6" t="n">
         <v>9.0</v>
       </c>
     </row>
@@ -19761,17 +19788,20 @@
         <v>14488.95</v>
       </c>
       <c r="H35" s="6" t="n">
+        <v>1614.81</v>
+      </c>
+      <c r="I35" s="6" t="n">
         <v>14488.95</v>
       </c>
-      <c r="I35" s="6" t="n">
+      <c r="J35" s="6" t="n">
         <v>1614.81</v>
       </c>
-      <c r="J35" s="5" t="inlineStr">
+      <c r="K35" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="K35" s="6" t="n">
+      <c r="L35" s="6" t="n">
         <v>8.0</v>
       </c>
     </row>
@@ -19806,17 +19836,20 @@
         <v>17169.29</v>
       </c>
       <c r="H36" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I36" s="6" t="n">
         <v>17169.29</v>
       </c>
-      <c r="I36" s="6" t="n">
+      <c r="J36" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J36" s="5" t="inlineStr">
+      <c r="K36" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K36" s="6" t="n">
+      <c r="L36" s="6" t="n">
         <v>5.0</v>
       </c>
     </row>
@@ -19851,17 +19884,20 @@
         <v>15885.27</v>
       </c>
       <c r="H37" s="6" t="n">
+        <v>-547.77</v>
+      </c>
+      <c r="I37" s="6" t="n">
         <v>15337.5</v>
       </c>
-      <c r="I37" s="6" t="n">
+      <c r="J37" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J37" s="5" t="inlineStr">
+      <c r="K37" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K37" s="6" t="n">
+      <c r="L37" s="6" t="n">
         <v>9.0</v>
       </c>
     </row>
@@ -19896,17 +19932,20 @@
         <v>13838.4</v>
       </c>
       <c r="H38" s="6" t="n">
+        <v>2767.68</v>
+      </c>
+      <c r="I38" s="6" t="n">
         <v>13838.4</v>
       </c>
-      <c r="I38" s="6" t="n">
+      <c r="J38" s="6" t="n">
         <v>2767.68</v>
       </c>
-      <c r="J38" s="5" t="inlineStr">
+      <c r="K38" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="K38" s="6" t="n">
+      <c r="L38" s="6" t="n">
         <v>5.0</v>
       </c>
     </row>
@@ -19941,17 +19980,20 @@
         <v>17989.92</v>
       </c>
       <c r="H39" s="6" t="n">
+        <v>-2767.68</v>
+      </c>
+      <c r="I39" s="6" t="n">
         <v>15222.24</v>
       </c>
-      <c r="I39" s="6" t="n">
+      <c r="J39" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J39" s="5" t="inlineStr">
+      <c r="K39" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K39" s="6" t="n">
+      <c r="L39" s="6" t="n">
         <v>5.0</v>
       </c>
     </row>
@@ -19986,17 +20028,20 @@
         <v>10825.92</v>
       </c>
       <c r="H40" s="6" t="n">
+        <v>-2686.08</v>
+      </c>
+      <c r="I40" s="6" t="n">
         <v>10825.92</v>
       </c>
-      <c r="I40" s="6" t="n">
+      <c r="J40" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J40" s="5" t="inlineStr">
+      <c r="K40" s="5" t="inlineStr">
         <is>
           <t>OVERPAID</t>
         </is>
       </c>
-      <c r="K40" s="6" t="n">
+      <c r="L40" s="6" t="n">
         <v>7.0</v>
       </c>
     </row>
@@ -20031,17 +20076,20 @@
         <v>25184.36</v>
       </c>
       <c r="H41" s="6" t="n">
+        <v>2686.08</v>
+      </c>
+      <c r="I41" s="6" t="n">
         <v>25184.36</v>
       </c>
-      <c r="I41" s="6" t="n">
+      <c r="J41" s="6" t="n">
         <v>2686.08</v>
       </c>
-      <c r="J41" s="5" t="inlineStr">
+      <c r="K41" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="K41" s="6" t="n">
+      <c r="L41" s="6" t="n">
         <v>9.0</v>
       </c>
     </row>
@@ -20076,17 +20124,20 @@
         <v>11335.68</v>
       </c>
       <c r="H42" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I42" s="6" t="n">
         <v>11335.68</v>
       </c>
-      <c r="I42" s="6" t="n">
+      <c r="J42" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J42" s="5" t="inlineStr">
+      <c r="K42" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K42" s="6" t="n">
+      <c r="L42" s="6" t="n">
         <v>4.0</v>
       </c>
     </row>
@@ -20121,17 +20172,20 @@
         <v>12343.07</v>
       </c>
       <c r="H43" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I43" s="6" t="n">
         <v>12343.07</v>
       </c>
-      <c r="I43" s="6" t="n">
+      <c r="J43" s="6" t="n">
         <v>-0.0</v>
       </c>
-      <c r="J43" s="5" t="inlineStr">
+      <c r="K43" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K43" s="6" t="n">
+      <c r="L43" s="6" t="n">
         <v>3.0</v>
       </c>
     </row>
@@ -20166,17 +20220,20 @@
         <v>15409.46</v>
       </c>
       <c r="H44" s="6" t="n">
+        <v>702.04</v>
+      </c>
+      <c r="I44" s="6" t="n">
         <v>15409.46</v>
       </c>
-      <c r="I44" s="6" t="n">
+      <c r="J44" s="6" t="n">
         <v>702.04</v>
       </c>
-      <c r="J44" s="5" t="inlineStr">
+      <c r="K44" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="K44" s="6" t="n">
+      <c r="L44" s="6" t="n">
         <v>4.0</v>
       </c>
     </row>
@@ -20211,17 +20268,20 @@
         <v>15140.69</v>
       </c>
       <c r="H45" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I45" s="6" t="n">
         <v>15140.69</v>
       </c>
-      <c r="I45" s="6" t="n">
+      <c r="J45" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J45" s="5" t="inlineStr">
+      <c r="K45" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K45" s="6" t="n">
+      <c r="L45" s="6" t="n">
         <v>4.0</v>
       </c>
     </row>
@@ -20256,17 +20316,20 @@
         <v>13806.77</v>
       </c>
       <c r="H46" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I46" s="6" t="n">
         <v>13806.77</v>
       </c>
-      <c r="I46" s="6" t="n">
+      <c r="J46" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J46" s="5" t="inlineStr">
+      <c r="K46" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K46" s="6" t="n">
+      <c r="L46" s="6" t="n">
         <v>4.0</v>
       </c>
     </row>
@@ -20301,17 +20364,20 @@
         <v>16964.84</v>
       </c>
       <c r="H47" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I47" s="6" t="n">
         <v>16964.84</v>
       </c>
-      <c r="I47" s="6" t="n">
+      <c r="J47" s="6" t="n">
         <v>-0.0</v>
       </c>
-      <c r="J47" s="5" t="inlineStr">
+      <c r="K47" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K47" s="6" t="n">
+      <c r="L47" s="6" t="n">
         <v>5.0</v>
       </c>
     </row>
@@ -20346,17 +20412,20 @@
         <v>13911.54</v>
       </c>
       <c r="H48" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I48" s="6" t="n">
         <v>13911.54</v>
       </c>
-      <c r="I48" s="6" t="n">
+      <c r="J48" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J48" s="5" t="inlineStr">
+      <c r="K48" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K48" s="6" t="n">
+      <c r="L48" s="6" t="n">
         <v>5.0</v>
       </c>
     </row>
@@ -20391,17 +20460,20 @@
         <v>12520.81</v>
       </c>
       <c r="H49" s="6" t="n">
+        <v>3245.76</v>
+      </c>
+      <c r="I49" s="6" t="n">
         <v>12520.81</v>
       </c>
-      <c r="I49" s="6" t="n">
+      <c r="J49" s="6" t="n">
         <v>3245.76</v>
       </c>
-      <c r="J49" s="5" t="inlineStr">
+      <c r="K49" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="K49" s="6" t="n">
+      <c r="L49" s="6" t="n">
         <v>5.0</v>
       </c>
     </row>
@@ -20436,17 +20508,20 @@
         <v>24801.28</v>
       </c>
       <c r="H50" s="6" t="n">
+        <v>-16774.3</v>
+      </c>
+      <c r="I50" s="6" t="n">
         <v>11272.74</v>
       </c>
-      <c r="I50" s="6" t="n">
+      <c r="J50" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J50" s="5" t="inlineStr">
+      <c r="K50" s="5" t="inlineStr">
         <is>
           <t>OVERPAID</t>
         </is>
       </c>
-      <c r="K50" s="6" t="n">
+      <c r="L50" s="6" t="n">
         <v>6.0</v>
       </c>
     </row>
@@ -20481,17 +20556,20 @@
         <v>16151.04</v>
       </c>
       <c r="H51" s="6" t="n">
+        <v>-2622.5</v>
+      </c>
+      <c r="I51" s="6" t="n">
         <v>13528.54</v>
       </c>
-      <c r="I51" s="6" t="n">
+      <c r="J51" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J51" s="5" t="inlineStr">
+      <c r="K51" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K51" s="6" t="n">
+      <c r="L51" s="6" t="n">
         <v>5.0</v>
       </c>
     </row>
@@ -20526,17 +20604,20 @@
         <v>14208.48</v>
       </c>
       <c r="H52" s="6" t="n">
+        <v>-2583.36</v>
+      </c>
+      <c r="I52" s="6" t="n">
         <v>11625.12</v>
       </c>
-      <c r="I52" s="6" t="n">
+      <c r="J52" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J52" s="5" t="inlineStr">
+      <c r="K52" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K52" s="6" t="n">
+      <c r="L52" s="6" t="n">
         <v>3.0</v>
       </c>
     </row>
@@ -20571,17 +20652,20 @@
         <v>18441.12</v>
       </c>
       <c r="H53" s="6" t="n">
+        <v>293.34</v>
+      </c>
+      <c r="I53" s="6" t="n">
         <v>18441.12</v>
       </c>
-      <c r="I53" s="6" t="n">
+      <c r="J53" s="6" t="n">
         <v>293.34</v>
       </c>
-      <c r="J53" s="5" t="inlineStr">
+      <c r="K53" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="K53" s="6" t="n">
+      <c r="L53" s="6" t="n">
         <v>7.0</v>
       </c>
     </row>
@@ -20616,17 +20700,20 @@
         <v>11105.31</v>
       </c>
       <c r="H54" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I54" s="6" t="n">
         <v>11105.31</v>
       </c>
-      <c r="I54" s="6" t="n">
+      <c r="J54" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J54" s="5" t="inlineStr">
+      <c r="K54" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K54" s="6" t="n">
+      <c r="L54" s="6" t="n">
         <v>6.0</v>
       </c>
     </row>
@@ -20661,17 +20748,20 @@
         <v>17634.86</v>
       </c>
       <c r="H55" s="6" t="n">
+        <v>-3772.33</v>
+      </c>
+      <c r="I55" s="6" t="n">
         <v>13862.53</v>
       </c>
-      <c r="I55" s="6" t="n">
+      <c r="J55" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J55" s="5" t="inlineStr">
+      <c r="K55" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K55" s="6" t="n">
+      <c r="L55" s="6" t="n">
         <v>4.0</v>
       </c>
     </row>
@@ -20706,17 +20796,20 @@
         <v>15395.18</v>
       </c>
       <c r="H56" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I56" s="6" t="n">
         <v>15395.18</v>
       </c>
-      <c r="I56" s="6" t="n">
+      <c r="J56" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J56" s="5" t="inlineStr">
+      <c r="K56" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K56" s="6" t="n">
+      <c r="L56" s="6" t="n">
         <v>5.0</v>
       </c>
     </row>
@@ -20751,17 +20844,20 @@
         <v>20232.18</v>
       </c>
       <c r="H57" s="6" t="n">
+        <v>-7597.32</v>
+      </c>
+      <c r="I57" s="6" t="n">
         <v>12634.86</v>
       </c>
-      <c r="I57" s="6" t="n">
+      <c r="J57" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J57" s="5" t="inlineStr">
+      <c r="K57" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K57" s="6" t="n">
+      <c r="L57" s="6" t="n">
         <v>4.0</v>
       </c>
     </row>
@@ -20796,17 +20892,20 @@
         <v>13862.03</v>
       </c>
       <c r="H58" s="6" t="n">
+        <v>4394.91</v>
+      </c>
+      <c r="I58" s="6" t="n">
         <v>13862.03</v>
       </c>
-      <c r="I58" s="6" t="n">
+      <c r="J58" s="6" t="n">
         <v>4394.91</v>
       </c>
-      <c r="J58" s="5" t="inlineStr">
+      <c r="K58" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="K58" s="6" t="n">
+      <c r="L58" s="6" t="n">
         <v>6.0</v>
       </c>
     </row>
@@ -20841,17 +20940,20 @@
         <v>20443.0</v>
       </c>
       <c r="H59" s="6" t="n">
+        <v>-5210.82</v>
+      </c>
+      <c r="I59" s="6" t="n">
         <v>15232.18</v>
       </c>
-      <c r="I59" s="6" t="n">
+      <c r="J59" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J59" s="5" t="inlineStr">
+      <c r="K59" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K59" s="6" t="n">
+      <c r="L59" s="6" t="n">
         <v>4.0</v>
       </c>
     </row>
@@ -20886,17 +20988,20 @@
         <v>22336.89</v>
       </c>
       <c r="H60" s="6" t="n">
+        <v>-6893.89</v>
+      </c>
+      <c r="I60" s="6" t="n">
         <v>15443.0</v>
       </c>
-      <c r="I60" s="6" t="n">
+      <c r="J60" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J60" s="5" t="inlineStr">
+      <c r="K60" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K60" s="6" t="n">
+      <c r="L60" s="6" t="n">
         <v>5.0</v>
       </c>
     </row>
@@ -20931,17 +21036,20 @@
         <v>19550.42</v>
       </c>
       <c r="H61" s="6" t="n">
+        <v>-4366.24</v>
+      </c>
+      <c r="I61" s="6" t="n">
         <v>15184.18</v>
       </c>
-      <c r="I61" s="6" t="n">
+      <c r="J61" s="6" t="n">
         <v>-0.0</v>
       </c>
-      <c r="J61" s="5" t="inlineStr">
+      <c r="K61" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K61" s="6" t="n">
+      <c r="L61" s="6" t="n">
         <v>5.0</v>
       </c>
     </row>
@@ -20977,18 +21085,23 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H62" s="6" t="n">
+      <c r="H62" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I62" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="I62" s="6" t="n">
+      <c r="J62" s="6" t="n">
         <v>15336.89</v>
       </c>
-      <c r="J62" s="5" t="inlineStr">
+      <c r="K62" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="K62" s="6" t="n">
+      <c r="L62" s="6" t="n">
         <v>5.0</v>
       </c>
     </row>
@@ -21024,18 +21137,23 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H63" s="6" t="n">
+      <c r="H63" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I63" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="I63" s="6" t="n">
+      <c r="J63" s="6" t="n">
         <v>14025.58</v>
       </c>
-      <c r="J63" s="5" t="inlineStr">
+      <c r="K63" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="K63" s="6" t="n">
+      <c r="L63" s="6" t="n">
         <v>7.0</v>
       </c>
     </row>
@@ -21071,18 +21189,23 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H64" s="6" t="n">
+      <c r="H64" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I64" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="I64" s="6" t="n">
+      <c r="J64" s="6" t="n">
         <v>12524.85</v>
       </c>
-      <c r="J64" s="5" t="inlineStr">
+      <c r="K64" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="K64" s="6" t="n">
+      <c r="L64" s="6" t="n">
         <v>4.0</v>
       </c>
     </row>
@@ -21117,17 +21240,20 @@
         <v>15816.63</v>
       </c>
       <c r="H65" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I65" s="6" t="n">
         <v>15816.63</v>
       </c>
-      <c r="I65" s="6" t="n">
+      <c r="J65" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J65" s="5" t="inlineStr">
+      <c r="K65" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K65" s="6" t="n">
+      <c r="L65" s="6" t="n">
         <v>4.0</v>
       </c>
     </row>
@@ -21150,31 +21276,32 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>00038846,00039812</t>
         </is>
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G66" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2025-05-22,2025-06-12</t>
+        </is>
+      </c>
+      <c r="G66" s="6" t="n">
+        <v>27895.66</v>
       </c>
       <c r="H66" s="6" t="n">
-        <v>0.0</v>
+        <v>-10320.82</v>
       </c>
       <c r="I66" s="6" t="n">
         <v>17574.84</v>
       </c>
-      <c r="J66" s="5" t="inlineStr">
-        <is>
-          <t>UNPAID</t>
-        </is>
-      </c>
-      <c r="K66" s="6" t="n">
+      <c r="J66" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K66" s="5" t="inlineStr">
+        <is>
+          <t>FULLY_SETTLED</t>
+        </is>
+      </c>
+      <c r="L66" s="6" t="n">
         <v>5.0</v>
       </c>
     </row>
@@ -21197,31 +21324,32 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>00039812</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G67" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2025-06-12</t>
+        </is>
+      </c>
+      <c r="G67" s="6" t="n">
+        <v>20557.69</v>
       </c>
       <c r="H67" s="6" t="n">
-        <v>0.0</v>
+        <v>-10236.87</v>
       </c>
       <c r="I67" s="6" t="n">
         <v>10320.82</v>
       </c>
-      <c r="J67" s="5" t="inlineStr">
-        <is>
-          <t>UNPAID</t>
-        </is>
-      </c>
-      <c r="K67" s="6" t="n">
+      <c r="J67" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K67" s="5" t="inlineStr">
+        <is>
+          <t>FULLY_SETTLED</t>
+        </is>
+      </c>
+      <c r="L67" s="6" t="n">
         <v>3.0</v>
       </c>
     </row>
@@ -21256,17 +21384,20 @@
         <v>11795.24</v>
       </c>
       <c r="H68" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I68" s="6" t="n">
         <v>11795.24</v>
       </c>
-      <c r="I68" s="6" t="n">
+      <c r="J68" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J68" s="5" t="inlineStr">
+      <c r="K68" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K68" s="6" t="n">
+      <c r="L68" s="6" t="n">
         <v>4.0</v>
       </c>
     </row>
@@ -21302,18 +21433,23 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H69" s="6" t="n">
+      <c r="H69" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I69" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="I69" s="6" t="n">
+      <c r="J69" s="6" t="n">
         <v>21724.53</v>
       </c>
-      <c r="J69" s="5" t="inlineStr">
+      <c r="K69" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="K69" s="6" t="n">
+      <c r="L69" s="6" t="n">
         <v>5.0</v>
       </c>
     </row>
@@ -21349,18 +21485,23 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H70" s="6" t="n">
+      <c r="H70" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I70" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="I70" s="6" t="n">
+      <c r="J70" s="6" t="n">
         <v>13342.37</v>
       </c>
-      <c r="J70" s="5" t="inlineStr">
+      <c r="K70" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="K70" s="6" t="n">
+      <c r="L70" s="6" t="n">
         <v>6.0</v>
       </c>
     </row>
@@ -21383,29 +21524,36 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t>00040746</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>2025-08-22</t>
-        </is>
-      </c>
-      <c r="G71" s="6" t="n">
-        <v>14579.44</v>
-      </c>
-      <c r="H71" s="6" t="n">
-        <v>14579.44</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H71" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I71" s="6" t="n">
-        <v>38.67</v>
-      </c>
-      <c r="J71" s="5" t="inlineStr">
-        <is>
-          <t>PARTIALLY_SETTLED</t>
-        </is>
-      </c>
-      <c r="K71" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J71" s="6" t="n">
+        <v>14618.11</v>
+      </c>
+      <c r="K71" s="5" t="inlineStr">
+        <is>
+          <t>UNPAID</t>
+        </is>
+      </c>
+      <c r="L71" s="6" t="n">
         <v>6.0</v>
       </c>
     </row>
@@ -21428,18 +21576,16 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>00040746</t>
         </is>
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G72" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2025-08-22</t>
+        </is>
+      </c>
+      <c r="G72" s="6" t="n">
+        <v>14579.44</v>
       </c>
       <c r="H72" s="6" t="n">
         <v>0.0</v>
@@ -21447,12 +21593,15 @@
       <c r="I72" s="6" t="n">
         <v>14579.44</v>
       </c>
-      <c r="J72" s="5" t="inlineStr">
-        <is>
-          <t>UNPAID</t>
-        </is>
-      </c>
-      <c r="K72" s="6" t="n">
+      <c r="J72" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K72" s="5" t="inlineStr">
+        <is>
+          <t>FULLY_SETTLED</t>
+        </is>
+      </c>
+      <c r="L72" s="6" t="n">
         <v>5.0</v>
       </c>
     </row>
@@ -21487,17 +21636,20 @@
         <v>16601.81</v>
       </c>
       <c r="H73" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I73" s="6" t="n">
         <v>16601.81</v>
       </c>
-      <c r="I73" s="6" t="n">
+      <c r="J73" s="6" t="n">
         <v>0.01</v>
       </c>
-      <c r="J73" s="5" t="inlineStr">
+      <c r="K73" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K73" s="6" t="n">
+      <c r="L73" s="6" t="n">
         <v>5.0</v>
       </c>
     </row>
@@ -21532,17 +21684,20 @@
         <v>13327.87</v>
       </c>
       <c r="H74" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I74" s="6" t="n">
         <v>13327.87</v>
       </c>
-      <c r="I74" s="6" t="n">
+      <c r="J74" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J74" s="5" t="inlineStr">
+      <c r="K74" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K74" s="6" t="n">
+      <c r="L74" s="6" t="n">
         <v>4.0</v>
       </c>
     </row>
@@ -21577,17 +21732,20 @@
         <v>13161.86</v>
       </c>
       <c r="H75" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I75" s="6" t="n">
         <v>13161.86</v>
       </c>
-      <c r="I75" s="6" t="n">
+      <c r="J75" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J75" s="5" t="inlineStr">
+      <c r="K75" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K75" s="6" t="n">
+      <c r="L75" s="6" t="n">
         <v>4.0</v>
       </c>
     </row>
@@ -21622,17 +21780,20 @@
         <v>15578.23</v>
       </c>
       <c r="H76" s="6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I76" s="6" t="n">
         <v>15578.23</v>
       </c>
-      <c r="I76" s="6" t="n">
+      <c r="J76" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="J76" s="5" t="inlineStr">
+      <c r="K76" s="5" t="inlineStr">
         <is>
           <t>FULLY_SETTLED</t>
         </is>
       </c>
-      <c r="K76" s="6" t="n">
+      <c r="L76" s="6" t="n">
         <v>5.0</v>
       </c>
     </row>
@@ -21668,18 +21829,23 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H77" s="6" t="n">
+      <c r="H77" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I77" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="I77" s="6" t="n">
+      <c r="J77" s="6" t="n">
         <v>11666.11</v>
       </c>
-      <c r="J77" s="5" t="inlineStr">
+      <c r="K77" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="K77" s="6" t="n">
+      <c r="L77" s="6" t="n">
         <v>6.0</v>
       </c>
     </row>
@@ -21715,18 +21881,23 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H78" s="6" t="n">
+      <c r="H78" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I78" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="I78" s="6" t="n">
+      <c r="J78" s="6" t="n">
         <v>14323.09</v>
       </c>
-      <c r="J78" s="5" t="inlineStr">
+      <c r="K78" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="K78" s="6" t="n">
+      <c r="L78" s="6" t="n">
         <v>6.0</v>
       </c>
     </row>
@@ -21762,18 +21933,23 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H79" s="6" t="n">
+      <c r="H79" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I79" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="I79" s="6" t="n">
+      <c r="J79" s="6" t="n">
         <v>10559.95</v>
       </c>
-      <c r="J79" s="5" t="inlineStr">
+      <c r="K79" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="K79" s="6" t="n">
+      <c r="L79" s="6" t="n">
         <v>3.0</v>
       </c>
     </row>
@@ -21808,17 +21984,20 @@
         <v>11666.12</v>
       </c>
       <c r="H80" s="6" t="n">
+        <v>271.44</v>
+      </c>
+      <c r="I80" s="6" t="n">
         <v>11666.12</v>
       </c>
-      <c r="I80" s="6" t="n">
+      <c r="J80" s="6" t="n">
         <v>271.44</v>
       </c>
-      <c r="J80" s="5" t="inlineStr">
+      <c r="K80" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY_SETTLED</t>
         </is>
       </c>
-      <c r="K80" s="6" t="n">
+      <c r="L80" s="6" t="n">
         <v>5.0</v>
       </c>
     </row>
@@ -21854,18 +22033,23 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H81" s="6" t="n">
+      <c r="H81" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I81" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="I81" s="6" t="n">
+      <c r="J81" s="6" t="n">
         <v>14303.99</v>
       </c>
-      <c r="J81" s="5" t="inlineStr">
+      <c r="K81" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="K81" s="6" t="n">
+      <c r="L81" s="6" t="n">
         <v>4.0</v>
       </c>
     </row>
@@ -21901,18 +22085,23 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H82" s="6" t="n">
+      <c r="H82" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I82" s="6" t="n">
         <v>0.0</v>
       </c>
-      <c r="I82" s="6" t="n">
+      <c r="J82" s="6" t="n">
         <v>21274.86</v>
       </c>
-      <c r="J82" s="5" t="inlineStr">
+      <c r="K82" s="5" t="inlineStr">
         <is>
           <t>UNPAID</t>
         </is>
       </c>
-      <c r="K82" s="6" t="n">
+      <c r="L82" s="6" t="n">
         <v>5.0</v>
       </c>
     </row>
@@ -21951,17 +22140,20 @@
         </is>
       </c>
       <c r="H83" s="6" t="n">
-        <v>836374.12</v>
+        <v>-56458.08</v>
       </c>
       <c r="I83" s="6" t="n">
-        <v>273153.18</v>
-      </c>
-      <c r="J83" s="5" t="inlineStr">
+        <v>864269.78</v>
+      </c>
+      <c r="J83" s="6" t="n">
+        <v>245257.52</v>
+      </c>
+      <c r="K83" s="5" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K83" s="5" t="inlineStr">
+      <c r="L83" s="5" t="inlineStr">
         <is>
           <t/>
         </is>

</xml_diff>

<commit_message>
JIM001: allocate doc 44555 to December 2025 (account-owner decision)
Closes the December-2025-vs-March-2026 dispute by explicit instruction,
not new evidence -- the raw ERP ledger still shows this payment untagged
to any invoice either way. December moves UNPAID -> FULLY_SETTLED
(1-cent rounding residual); March 2026 reverts to genuinely UNPAID in
full. Recorded as evidence_status ASSERTED (decision), Tier 3 -- not
PROVEN, unlike doc 40746's Tier 2 resolution. Updated the bridge review,
legal handoff checklist, project history, and both reconciliation
workbooks to match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012bZD667N5ecomW85qEfDtW
</commit_message>
<xml_diff>
--- a/analysis/debtors/JIM001/reports/JIM001_LPG_Reconciliation_v4.1.xlsx
+++ b/analysis/debtors/JIM001/reports/JIM001_LPG_Reconciliation_v4.1.xlsx
@@ -20,11 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="R#,##0.00;[Red]-R#,##0.00;&quot;—&quot;"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -153,7 +152,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -211,7 +210,8 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -306,12 +306,12 @@
 <file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>Claude (JIM001 bridge review)</author>
+    <author>Claude</author>
   </authors>
   <commentList>
     <comment ref="D30" authorId="0" shapeId="0">
       <text>
-        <t>R0.01 variance (11,666.12 vs 11,666.11), same rounding tolerance treated as exact elsewhere in this sheet (e.g. docs 8420, 41664). ASSERTED via aggregate exact-sum match, not PROVEN -- no remittance advice exists for JIM001. Contradicts the unconfirmed ERP-ledger invoice split (allocation_edges.csv AL-0359-AL-0361) which points to March 2026 instead. See JIM001_Exact_Sum_Bridge_Review_2026-09-13.md SS5.</t>
+        <t>R0.01 variance (11,666.12 vs 11,666.11), same rounding tolerance treated as exact elsewhere in this sheet (e.g. docs 8420, 41664). CLOSED BY ACCOUNT-OWNER DECISION (2026-09-14): allocated to December 2025 to settle the December-vs-March-2026 dispute ahead of legal handoff. Not independently proven -- the raw ERP ledger (raw/DEBENQ_CURRENT.TXT) shows this payment untagged to any invoice, December included, and the competing March-2026 invoice-level split (allocation_edges.csv AL-0359-AL-0361) is confirmed fictitious (does not exist in the real ERP either). Evidence status: ASSERTED (decision), Tier 3 -- not PROVEN. See JIM001_Exact_Sum_Bridge_Review_2026-09-13.md SS5.</t>
       </text>
     </comment>
   </commentList>
@@ -18840,7 +18840,7 @@
         <v>10874.96</v>
       </c>
       <c r="J14" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
@@ -19232,7 +19232,7 @@
         <v>12222.9</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
@@ -20244,7 +20244,7 @@
         <v>12343.07</v>
       </c>
       <c r="J43" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="K43" s="5" t="inlineStr">
         <is>
@@ -20436,7 +20436,7 @@
         <v>16964.84</v>
       </c>
       <c r="J47" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="K47" s="5" t="inlineStr">
         <is>
@@ -21108,7 +21108,7 @@
         <v>15184.18</v>
       </c>
       <c r="J61" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="K61" s="5" t="inlineStr">
         <is>
@@ -21882,18 +21882,16 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>00044555</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G77" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="n">
+        <v>11666.12</v>
       </c>
       <c r="H77" s="5" t="inlineStr">
         <is>
@@ -22038,16 +22036,18 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t>00044555</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
-        </is>
-      </c>
-      <c r="G80" s="6" t="n">
-        <v>11666.12</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G80" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="H80" s="6" t="n">
         <v>271.44</v>
@@ -22439,7 +22439,7 @@
     <row r="17">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t>2. Doc 44555 — UNRESOLVED: untagged in the real ERP</t>
+          <t>2. Doc 44555 — untagged in the real ERP; CLOSED BY ACCOUNT-OWNER DECISION (December 2025)</t>
         </is>
       </c>
     </row>
@@ -22496,7 +22496,7 @@
     <row r="21" ht="42" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>Conclusion: allocation_edges.csv's claimed split to 3 named March-2026 invoices (AL-0359–AL-0361) does NOT exist in the real ERP -- confirmed fictitious, not merely unconfirmed. The competing December-2025 aggregate-total-match reading is now the only one with any support, but it was never ERP-tagged either -- still ASSERTED, not PROVEN. Needs an actual remittance advice to settle.</t>
+          <t>Finding: allocation_edges.csv's claimed split to 3 named March-2026 invoices (AL-0359–AL-0361) does NOT exist in the real ERP -- confirmed fictitious, not merely unconfirmed. Neither December 2025 nor March 2026 is ERP-tagged; the ERP simply doesn't tag this payment at all. Update (2026-09-14): closed by explicit account-owner decision, not by new evidence -- doc 44555 is now allocated to December 2025 (the only reading with any support, via the aggregate exact-sum match) to settle this ahead of legal handoff. Recorded as ASSERTED (decision), Tier 3, NOT PROVEN. Revisit if a remittance advice for doc 44555 ever surfaces.</t>
         </is>
       </c>
     </row>
@@ -22603,7 +22603,7 @@
           <t>Tie-out %</t>
         </is>
       </c>
-      <c r="C36" s="27">
+      <c r="C36" s="28">
         <f>1-ABS(C35)/C28</f>
         <v/>
       </c>

</xml_diff>